<commit_message>
dashboard update 2026-10-18 (laptop)
</commit_message>
<xml_diff>
--- a/data/nowcast/DE_data_inspect_noreal_sent_levels_auth.xlsx
+++ b/data/nowcast/DE_data_inspect_noreal_sent_levels_auth.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,24 +45,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,64 +421,64 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>GDPyoy</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>EURIBOR 3M</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EcSent</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>IPall</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>CONSindex</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>retail</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>unemployment</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>HICP</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Brent</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>STOXX</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>31078</v>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -509,7 +495,7 @@
       <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>31106</v>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -526,7 +512,7 @@
       <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>31137</v>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -543,7 +529,7 @@
       <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>31167</v>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -560,7 +546,7 @@
       <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>31198</v>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -577,7 +563,7 @@
       <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>31228</v>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -594,7 +580,7 @@
       <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>31259</v>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -611,7 +597,7 @@
       <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>31290</v>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -628,7 +614,7 @@
       <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>31320</v>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -645,7 +631,7 @@
       <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>31351</v>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -662,7 +648,7 @@
       <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>31381</v>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -679,7 +665,7 @@
       <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>31412</v>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -696,7 +682,7 @@
       <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>31443</v>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -713,7 +699,7 @@
       <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>31471</v>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -730,7 +716,7 @@
       <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>31502</v>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -747,7 +733,7 @@
       <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>31532</v>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -764,7 +750,7 @@
       <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>31563</v>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -781,7 +767,7 @@
       <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>31593</v>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -798,7 +784,7 @@
       <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>31624</v>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -815,7 +801,7 @@
       <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>31655</v>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -832,7 +818,7 @@
       <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>31685</v>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -849,7 +835,7 @@
       <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>31716</v>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -866,7 +852,7 @@
       <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>31746</v>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -883,7 +869,7 @@
       <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>31777</v>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -900,7 +886,7 @@
       <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="1" t="n">
         <v>31808</v>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -917,7 +903,7 @@
       <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="1" t="n">
         <v>31836</v>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -934,7 +920,7 @@
       <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="1" t="n">
         <v>31867</v>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -951,7 +937,7 @@
       <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="1" t="n">
         <v>31897</v>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -968,7 +954,7 @@
       <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="1" t="n">
         <v>31928</v>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -985,7 +971,7 @@
       <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>31958</v>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1002,7 +988,7 @@
       <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="1" t="n">
         <v>31989</v>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1019,7 +1005,7 @@
       <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="1" t="n">
         <v>32020</v>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1036,7 +1022,7 @@
       <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="1" t="n">
         <v>32050</v>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1053,7 +1039,7 @@
       <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="1" t="n">
         <v>32081</v>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1070,7 +1056,7 @@
       <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="1" t="n">
         <v>32111</v>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1087,7 +1073,7 @@
       <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="1" t="n">
         <v>32142</v>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -1104,7 +1090,7 @@
       <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="1" t="n">
         <v>32173</v>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -1121,7 +1107,7 @@
       <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="1" t="n">
         <v>32202</v>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -1138,7 +1124,7 @@
       <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="1" t="n">
         <v>32233</v>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -1155,7 +1141,7 @@
       <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="1" t="n">
         <v>32263</v>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -1172,7 +1158,7 @@
       <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="1" t="n">
         <v>32294</v>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -1189,7 +1175,7 @@
       <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="1" t="n">
         <v>32324</v>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -1206,7 +1192,7 @@
       <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="1" t="n">
         <v>32355</v>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1223,7 +1209,7 @@
       <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="1" t="n">
         <v>32386</v>
       </c>
       <c r="B45" t="inlineStr"/>
@@ -1240,7 +1226,7 @@
       <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>32416</v>
       </c>
       <c r="B46" t="inlineStr"/>
@@ -1257,7 +1243,7 @@
       <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="1" t="n">
         <v>32447</v>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -1274,7 +1260,7 @@
       <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="1" t="n">
         <v>32477</v>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -1291,7 +1277,7 @@
       <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="1" t="n">
         <v>32508</v>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -1308,7 +1294,7 @@
       <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>32539</v>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -1325,7 +1311,7 @@
       <c r="K50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="1" t="n">
         <v>32567</v>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -1342,7 +1328,7 @@
       <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="1" t="n">
         <v>32598</v>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -1359,7 +1345,7 @@
       <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="1" t="n">
         <v>32628</v>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -1376,7 +1362,7 @@
       <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="1" t="n">
         <v>32659</v>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -1393,7 +1379,7 @@
       <c r="K54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="1" t="n">
         <v>32689</v>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -1410,7 +1396,7 @@
       <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="1" t="n">
         <v>32720</v>
       </c>
       <c r="B56" t="inlineStr"/>
@@ -1427,7 +1413,7 @@
       <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="1" t="n">
         <v>32751</v>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -1444,7 +1430,7 @@
       <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="1" t="n">
         <v>32781</v>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -1461,7 +1447,7 @@
       <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="1" t="n">
         <v>32812</v>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -1478,7 +1464,7 @@
       <c r="K59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="1" t="n">
         <v>32842</v>
       </c>
       <c r="B60" t="inlineStr"/>
@@ -1495,7 +1481,7 @@
       <c r="K60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>32873</v>
       </c>
       <c r="B61" t="inlineStr"/>
@@ -1512,7 +1498,7 @@
       <c r="K61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="1" t="n">
         <v>32904</v>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -1529,7 +1515,7 @@
       <c r="K62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="1" t="n">
         <v>32932</v>
       </c>
       <c r="B63" t="inlineStr"/>
@@ -1546,7 +1532,7 @@
       <c r="K63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="1" t="n">
         <v>32963</v>
       </c>
       <c r="B64" t="inlineStr"/>
@@ -1563,7 +1549,7 @@
       <c r="K64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="1" t="n">
         <v>32993</v>
       </c>
       <c r="B65" t="inlineStr"/>
@@ -1580,7 +1566,7 @@
       <c r="K65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="1" t="n">
         <v>33024</v>
       </c>
       <c r="B66" t="inlineStr"/>
@@ -1597,7 +1583,7 @@
       <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="1" t="n">
         <v>33054</v>
       </c>
       <c r="B67" t="inlineStr"/>
@@ -1614,7 +1600,7 @@
       <c r="K67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="1" t="n">
         <v>33085</v>
       </c>
       <c r="B68" t="inlineStr"/>
@@ -1631,7 +1617,7 @@
       <c r="K68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="1" t="n">
         <v>33116</v>
       </c>
       <c r="B69" t="inlineStr"/>
@@ -1648,7 +1634,7 @@
       <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="1" t="n">
         <v>33146</v>
       </c>
       <c r="B70" t="inlineStr"/>
@@ -1665,7 +1651,7 @@
       <c r="K70" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="1" t="n">
         <v>33177</v>
       </c>
       <c r="B71" t="inlineStr"/>
@@ -1682,7 +1668,7 @@
       <c r="K71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="1" t="n">
         <v>33207</v>
       </c>
       <c r="B72" t="inlineStr"/>
@@ -1699,7 +1685,7 @@
       <c r="K72" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="1" t="n">
         <v>33238</v>
       </c>
       <c r="B73" t="inlineStr"/>
@@ -1716,7 +1702,7 @@
       <c r="K73" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="1" t="n">
         <v>33269</v>
       </c>
       <c r="B74" t="inlineStr"/>
@@ -1739,7 +1725,7 @@
       <c r="K74" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="1" t="n">
         <v>33297</v>
       </c>
       <c r="B75" t="inlineStr"/>
@@ -1762,7 +1748,7 @@
       <c r="K75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="1" t="n">
         <v>33328</v>
       </c>
       <c r="B76" t="n">
@@ -1787,7 +1773,7 @@
       <c r="K76" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="1" t="n">
         <v>33358</v>
       </c>
       <c r="B77" t="inlineStr"/>
@@ -1810,7 +1796,7 @@
       <c r="K77" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="1" t="n">
         <v>33389</v>
       </c>
       <c r="B78" t="inlineStr"/>
@@ -1833,7 +1819,7 @@
       <c r="K78" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="1" t="n">
         <v>33419</v>
       </c>
       <c r="B79" t="n">
@@ -1858,7 +1844,7 @@
       <c r="K79" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="1" t="n">
         <v>33450</v>
       </c>
       <c r="B80" t="inlineStr"/>
@@ -1881,7 +1867,7 @@
       <c r="K80" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="1" t="n">
         <v>33481</v>
       </c>
       <c r="B81" t="inlineStr"/>
@@ -1904,7 +1890,7 @@
       <c r="K81" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="1" t="n">
         <v>33511</v>
       </c>
       <c r="B82" t="n">
@@ -1929,7 +1915,7 @@
       <c r="K82" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="1" t="n">
         <v>33542</v>
       </c>
       <c r="B83" t="inlineStr"/>
@@ -1952,7 +1938,7 @@
       <c r="K83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="1" t="n">
         <v>33572</v>
       </c>
       <c r="B84" t="inlineStr"/>
@@ -1975,7 +1961,7 @@
       <c r="K84" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="1" t="n">
         <v>33603</v>
       </c>
       <c r="B85" t="n">
@@ -2000,7 +1986,7 @@
       <c r="K85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="1" t="n">
         <v>33634</v>
       </c>
       <c r="B86" t="inlineStr"/>
@@ -2023,7 +2009,7 @@
       <c r="K86" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="1" t="n">
         <v>33663</v>
       </c>
       <c r="B87" t="inlineStr"/>
@@ -2046,7 +2032,7 @@
       <c r="K87" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="1" t="n">
         <v>33694</v>
       </c>
       <c r="B88" t="n">
@@ -2071,7 +2057,7 @@
       <c r="K88" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="1" t="n">
         <v>33724</v>
       </c>
       <c r="B89" t="inlineStr"/>
@@ -2094,7 +2080,7 @@
       <c r="K89" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="1" t="n">
         <v>33755</v>
       </c>
       <c r="B90" t="inlineStr"/>
@@ -2117,7 +2103,7 @@
       <c r="K90" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="1" t="n">
         <v>33785</v>
       </c>
       <c r="B91" t="n">
@@ -2142,7 +2128,7 @@
       <c r="K91" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="1" t="n">
         <v>33816</v>
       </c>
       <c r="B92" t="inlineStr"/>
@@ -2165,7 +2151,7 @@
       <c r="K92" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="1" t="n">
         <v>33847</v>
       </c>
       <c r="B93" t="inlineStr"/>
@@ -2188,7 +2174,7 @@
       <c r="K93" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n">
+      <c r="A94" s="1" t="n">
         <v>33877</v>
       </c>
       <c r="B94" t="n">
@@ -2213,7 +2199,7 @@
       <c r="K94" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n">
+      <c r="A95" s="1" t="n">
         <v>33908</v>
       </c>
       <c r="B95" t="inlineStr"/>
@@ -2236,7 +2222,7 @@
       <c r="K95" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="1" t="n">
         <v>33938</v>
       </c>
       <c r="B96" t="inlineStr"/>
@@ -2259,7 +2245,7 @@
       <c r="K96" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n">
+      <c r="A97" s="1" t="n">
         <v>33969</v>
       </c>
       <c r="B97" t="n">
@@ -2284,7 +2270,7 @@
       <c r="K97" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="1" t="n">
         <v>34000</v>
       </c>
       <c r="B98" t="inlineStr"/>
@@ -2307,7 +2293,7 @@
       <c r="K98" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="1" t="n">
         <v>34028</v>
       </c>
       <c r="B99" t="inlineStr"/>
@@ -2330,7 +2316,7 @@
       <c r="K99" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="1" t="n">
         <v>34059</v>
       </c>
       <c r="B100" t="n">
@@ -2355,7 +2341,7 @@
       <c r="K100" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="1" t="n">
         <v>34089</v>
       </c>
       <c r="B101" t="inlineStr"/>
@@ -2378,7 +2364,7 @@
       <c r="K101" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n">
+      <c r="A102" s="1" t="n">
         <v>34120</v>
       </c>
       <c r="B102" t="inlineStr"/>
@@ -2401,7 +2387,7 @@
       <c r="K102" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n">
+      <c r="A103" s="1" t="n">
         <v>34150</v>
       </c>
       <c r="B103" t="n">
@@ -2426,7 +2412,7 @@
       <c r="K103" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n">
+      <c r="A104" s="1" t="n">
         <v>34181</v>
       </c>
       <c r="B104" t="inlineStr"/>
@@ -2449,7 +2435,7 @@
       <c r="K104" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n">
+      <c r="A105" s="1" t="n">
         <v>34212</v>
       </c>
       <c r="B105" t="inlineStr"/>
@@ -2472,7 +2458,7 @@
       <c r="K105" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n">
+      <c r="A106" s="1" t="n">
         <v>34242</v>
       </c>
       <c r="B106" t="n">
@@ -2497,7 +2483,7 @@
       <c r="K106" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n">
+      <c r="A107" s="1" t="n">
         <v>34273</v>
       </c>
       <c r="B107" t="inlineStr"/>
@@ -2520,7 +2506,7 @@
       <c r="K107" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n">
+      <c r="A108" s="1" t="n">
         <v>34303</v>
       </c>
       <c r="B108" t="inlineStr"/>
@@ -2543,7 +2529,7 @@
       <c r="K108" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n">
+      <c r="A109" s="1" t="n">
         <v>34334</v>
       </c>
       <c r="B109" t="n">
@@ -2568,7 +2554,7 @@
       <c r="K109" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n">
+      <c r="A110" s="1" t="n">
         <v>34365</v>
       </c>
       <c r="B110" t="inlineStr"/>
@@ -2595,7 +2581,7 @@
       <c r="K110" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n">
+      <c r="A111" s="1" t="n">
         <v>34393</v>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -2622,7 +2608,7 @@
       <c r="K111" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n">
+      <c r="A112" s="1" t="n">
         <v>34424</v>
       </c>
       <c r="B112" t="n">
@@ -2651,7 +2637,7 @@
       <c r="K112" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n">
+      <c r="A113" s="1" t="n">
         <v>34454</v>
       </c>
       <c r="B113" t="inlineStr"/>
@@ -2678,7 +2664,7 @@
       <c r="K113" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n">
+      <c r="A114" s="1" t="n">
         <v>34485</v>
       </c>
       <c r="B114" t="inlineStr"/>
@@ -2705,7 +2691,7 @@
       <c r="K114" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n">
+      <c r="A115" s="1" t="n">
         <v>34515</v>
       </c>
       <c r="B115" t="n">
@@ -2734,7 +2720,7 @@
       <c r="K115" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n">
+      <c r="A116" s="1" t="n">
         <v>34546</v>
       </c>
       <c r="B116" t="inlineStr"/>
@@ -2761,7 +2747,7 @@
       <c r="K116" t="inlineStr"/>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n">
+      <c r="A117" s="1" t="n">
         <v>34577</v>
       </c>
       <c r="B117" t="inlineStr"/>
@@ -2788,7 +2774,7 @@
       <c r="K117" t="inlineStr"/>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n">
+      <c r="A118" s="1" t="n">
         <v>34607</v>
       </c>
       <c r="B118" t="n">
@@ -2817,7 +2803,7 @@
       <c r="K118" t="inlineStr"/>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n">
+      <c r="A119" s="1" t="n">
         <v>34638</v>
       </c>
       <c r="B119" t="inlineStr"/>
@@ -2844,7 +2830,7 @@
       <c r="K119" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n">
+      <c r="A120" s="1" t="n">
         <v>34668</v>
       </c>
       <c r="B120" t="inlineStr"/>
@@ -2871,7 +2857,7 @@
       <c r="K120" t="inlineStr"/>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n">
+      <c r="A121" s="1" t="n">
         <v>34699</v>
       </c>
       <c r="B121" t="n">
@@ -2900,7 +2886,7 @@
       <c r="K121" t="inlineStr"/>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n">
+      <c r="A122" s="1" t="n">
         <v>34730</v>
       </c>
       <c r="B122" t="inlineStr"/>
@@ -2927,7 +2913,7 @@
       <c r="K122" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n">
+      <c r="A123" s="1" t="n">
         <v>34758</v>
       </c>
       <c r="B123" t="inlineStr"/>
@@ -2954,7 +2940,7 @@
       <c r="K123" t="inlineStr"/>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n">
+      <c r="A124" s="1" t="n">
         <v>34789</v>
       </c>
       <c r="B124" t="n">
@@ -2983,7 +2969,7 @@
       <c r="K124" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n">
+      <c r="A125" s="1" t="n">
         <v>34819</v>
       </c>
       <c r="B125" t="inlineStr"/>
@@ -3010,7 +2996,7 @@
       <c r="K125" t="inlineStr"/>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" s="1" t="n">
         <v>34850</v>
       </c>
       <c r="B126" t="inlineStr"/>
@@ -3037,7 +3023,7 @@
       <c r="K126" t="inlineStr"/>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n">
+      <c r="A127" s="1" t="n">
         <v>34880</v>
       </c>
       <c r="B127" t="n">
@@ -3066,7 +3052,7 @@
       <c r="K127" t="inlineStr"/>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n">
+      <c r="A128" s="1" t="n">
         <v>34911</v>
       </c>
       <c r="B128" t="inlineStr"/>
@@ -3093,7 +3079,7 @@
       <c r="K128" t="inlineStr"/>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n">
+      <c r="A129" s="1" t="n">
         <v>34942</v>
       </c>
       <c r="B129" t="inlineStr"/>
@@ -3120,7 +3106,7 @@
       <c r="K129" t="inlineStr"/>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n">
+      <c r="A130" s="1" t="n">
         <v>34972</v>
       </c>
       <c r="B130" t="n">
@@ -3149,7 +3135,7 @@
       <c r="K130" t="inlineStr"/>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n">
+      <c r="A131" s="1" t="n">
         <v>35003</v>
       </c>
       <c r="B131" t="inlineStr"/>
@@ -3176,7 +3162,7 @@
       <c r="K131" t="inlineStr"/>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" s="1" t="n">
         <v>35033</v>
       </c>
       <c r="B132" t="inlineStr"/>
@@ -3203,7 +3189,7 @@
       <c r="K132" t="inlineStr"/>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" s="1" t="n">
         <v>35064</v>
       </c>
       <c r="B133" t="n">
@@ -3232,7 +3218,7 @@
       <c r="K133" t="inlineStr"/>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n">
+      <c r="A134" s="1" t="n">
         <v>35095</v>
       </c>
       <c r="B134" t="inlineStr"/>
@@ -3261,7 +3247,7 @@
       <c r="K134" t="inlineStr"/>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n">
+      <c r="A135" s="1" t="n">
         <v>35124</v>
       </c>
       <c r="B135" t="inlineStr"/>
@@ -3290,7 +3276,7 @@
       <c r="K135" t="inlineStr"/>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="1" t="n">
         <v>35155</v>
       </c>
       <c r="B136" t="n">
@@ -3321,7 +3307,7 @@
       <c r="K136" t="inlineStr"/>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="1" t="n">
         <v>35185</v>
       </c>
       <c r="B137" t="inlineStr"/>
@@ -3350,7 +3336,7 @@
       <c r="K137" t="inlineStr"/>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="1" t="n">
         <v>35216</v>
       </c>
       <c r="B138" t="inlineStr"/>
@@ -3379,7 +3365,7 @@
       <c r="K138" t="inlineStr"/>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n">
+      <c r="A139" s="1" t="n">
         <v>35246</v>
       </c>
       <c r="B139" t="n">
@@ -3410,7 +3396,7 @@
       <c r="K139" t="inlineStr"/>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n">
+      <c r="A140" s="1" t="n">
         <v>35277</v>
       </c>
       <c r="B140" t="inlineStr"/>
@@ -3439,7 +3425,7 @@
       <c r="K140" t="inlineStr"/>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n">
+      <c r="A141" s="1" t="n">
         <v>35308</v>
       </c>
       <c r="B141" t="inlineStr"/>
@@ -3468,7 +3454,7 @@
       <c r="K141" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n">
+      <c r="A142" s="1" t="n">
         <v>35338</v>
       </c>
       <c r="B142" t="n">
@@ -3499,7 +3485,7 @@
       <c r="K142" t="inlineStr"/>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n">
+      <c r="A143" s="1" t="n">
         <v>35369</v>
       </c>
       <c r="B143" t="inlineStr"/>
@@ -3528,7 +3514,7 @@
       <c r="K143" t="inlineStr"/>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n">
+      <c r="A144" s="1" t="n">
         <v>35399</v>
       </c>
       <c r="B144" t="inlineStr"/>
@@ -3557,7 +3543,7 @@
       <c r="K144" t="inlineStr"/>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n">
+      <c r="A145" s="1" t="n">
         <v>35430</v>
       </c>
       <c r="B145" t="n">
@@ -3588,7 +3574,7 @@
       <c r="K145" t="inlineStr"/>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n">
+      <c r="A146" s="1" t="n">
         <v>35461</v>
       </c>
       <c r="B146" t="inlineStr"/>
@@ -3617,7 +3603,7 @@
       <c r="K146" t="inlineStr"/>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n">
+      <c r="A147" s="1" t="n">
         <v>35489</v>
       </c>
       <c r="B147" t="inlineStr"/>
@@ -3646,7 +3632,7 @@
       <c r="K147" t="inlineStr"/>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n">
+      <c r="A148" s="1" t="n">
         <v>35520</v>
       </c>
       <c r="B148" t="n">
@@ -3677,7 +3663,7 @@
       <c r="K148" t="inlineStr"/>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n">
+      <c r="A149" s="1" t="n">
         <v>35550</v>
       </c>
       <c r="B149" t="inlineStr"/>
@@ -3706,7 +3692,7 @@
       <c r="K149" t="inlineStr"/>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n">
+      <c r="A150" s="1" t="n">
         <v>35581</v>
       </c>
       <c r="B150" t="inlineStr"/>
@@ -3735,7 +3721,7 @@
       <c r="K150" t="inlineStr"/>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n">
+      <c r="A151" s="1" t="n">
         <v>35611</v>
       </c>
       <c r="B151" t="n">
@@ -3766,7 +3752,7 @@
       <c r="K151" t="inlineStr"/>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n">
+      <c r="A152" s="1" t="n">
         <v>35642</v>
       </c>
       <c r="B152" t="inlineStr"/>
@@ -3795,7 +3781,7 @@
       <c r="K152" t="inlineStr"/>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n">
+      <c r="A153" s="1" t="n">
         <v>35673</v>
       </c>
       <c r="B153" t="inlineStr"/>
@@ -3824,7 +3810,7 @@
       <c r="K153" t="inlineStr"/>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n">
+      <c r="A154" s="1" t="n">
         <v>35703</v>
       </c>
       <c r="B154" t="n">
@@ -3855,7 +3841,7 @@
       <c r="K154" t="inlineStr"/>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n">
+      <c r="A155" s="1" t="n">
         <v>35734</v>
       </c>
       <c r="B155" t="inlineStr"/>
@@ -3884,7 +3870,7 @@
       <c r="K155" t="inlineStr"/>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n">
+      <c r="A156" s="1" t="n">
         <v>35764</v>
       </c>
       <c r="B156" t="inlineStr"/>
@@ -3913,7 +3899,7 @@
       <c r="K156" t="inlineStr"/>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n">
+      <c r="A157" s="1" t="n">
         <v>35795</v>
       </c>
       <c r="B157" t="n">
@@ -3944,7 +3930,7 @@
       <c r="K157" t="inlineStr"/>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n">
+      <c r="A158" s="1" t="n">
         <v>35826</v>
       </c>
       <c r="B158" t="inlineStr"/>
@@ -3973,7 +3959,7 @@
       <c r="K158" t="inlineStr"/>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n">
+      <c r="A159" s="1" t="n">
         <v>35854</v>
       </c>
       <c r="B159" t="inlineStr"/>
@@ -4002,7 +3988,7 @@
       <c r="K159" t="inlineStr"/>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n">
+      <c r="A160" s="1" t="n">
         <v>35885</v>
       </c>
       <c r="B160" t="n">
@@ -4033,7 +4019,7 @@
       <c r="K160" t="inlineStr"/>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n">
+      <c r="A161" s="1" t="n">
         <v>35915</v>
       </c>
       <c r="B161" t="inlineStr"/>
@@ -4062,7 +4048,7 @@
       <c r="K161" t="inlineStr"/>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n">
+      <c r="A162" s="1" t="n">
         <v>35946</v>
       </c>
       <c r="B162" t="inlineStr"/>
@@ -4091,7 +4077,7 @@
       <c r="K162" t="inlineStr"/>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n">
+      <c r="A163" s="1" t="n">
         <v>35976</v>
       </c>
       <c r="B163" t="n">
@@ -4122,7 +4108,7 @@
       <c r="K163" t="inlineStr"/>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n">
+      <c r="A164" s="1" t="n">
         <v>36007</v>
       </c>
       <c r="B164" t="inlineStr"/>
@@ -4151,7 +4137,7 @@
       <c r="K164" t="inlineStr"/>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n">
+      <c r="A165" s="1" t="n">
         <v>36038</v>
       </c>
       <c r="B165" t="inlineStr"/>
@@ -4180,7 +4166,7 @@
       <c r="K165" t="inlineStr"/>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n">
+      <c r="A166" s="1" t="n">
         <v>36068</v>
       </c>
       <c r="B166" t="n">
@@ -4211,7 +4197,7 @@
       <c r="K166" t="inlineStr"/>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n">
+      <c r="A167" s="1" t="n">
         <v>36099</v>
       </c>
       <c r="B167" t="inlineStr"/>
@@ -4240,7 +4226,7 @@
       <c r="K167" t="inlineStr"/>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n">
+      <c r="A168" s="1" t="n">
         <v>36129</v>
       </c>
       <c r="B168" t="inlineStr"/>
@@ -4269,7 +4255,7 @@
       <c r="K168" t="inlineStr"/>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n">
+      <c r="A169" s="1" t="n">
         <v>36160</v>
       </c>
       <c r="B169" t="n">
@@ -4300,7 +4286,7 @@
       <c r="K169" t="inlineStr"/>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n">
+      <c r="A170" s="1" t="n">
         <v>36191</v>
       </c>
       <c r="B170" t="inlineStr"/>
@@ -4331,7 +4317,7 @@
       <c r="K170" t="inlineStr"/>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n">
+      <c r="A171" s="1" t="n">
         <v>36219</v>
       </c>
       <c r="B171" t="inlineStr"/>
@@ -4362,7 +4348,7 @@
       <c r="K171" t="inlineStr"/>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n">
+      <c r="A172" s="1" t="n">
         <v>36250</v>
       </c>
       <c r="B172" t="n">
@@ -4395,7 +4381,7 @@
       <c r="K172" t="inlineStr"/>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n">
+      <c r="A173" s="1" t="n">
         <v>36280</v>
       </c>
       <c r="B173" t="inlineStr"/>
@@ -4426,7 +4412,7 @@
       <c r="K173" t="inlineStr"/>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n">
+      <c r="A174" s="1" t="n">
         <v>36311</v>
       </c>
       <c r="B174" t="inlineStr"/>
@@ -4457,7 +4443,7 @@
       <c r="K174" t="inlineStr"/>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n">
+      <c r="A175" s="1" t="n">
         <v>36341</v>
       </c>
       <c r="B175" t="n">
@@ -4490,7 +4476,7 @@
       <c r="K175" t="inlineStr"/>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n">
+      <c r="A176" s="1" t="n">
         <v>36372</v>
       </c>
       <c r="B176" t="inlineStr"/>
@@ -4521,7 +4507,7 @@
       <c r="K176" t="inlineStr"/>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n">
+      <c r="A177" s="1" t="n">
         <v>36403</v>
       </c>
       <c r="B177" t="inlineStr"/>
@@ -4552,7 +4538,7 @@
       <c r="K177" t="inlineStr"/>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n">
+      <c r="A178" s="1" t="n">
         <v>36433</v>
       </c>
       <c r="B178" t="n">
@@ -4585,7 +4571,7 @@
       <c r="K178" t="inlineStr"/>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n">
+      <c r="A179" s="1" t="n">
         <v>36464</v>
       </c>
       <c r="B179" t="inlineStr"/>
@@ -4616,7 +4602,7 @@
       <c r="K179" t="inlineStr"/>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n">
+      <c r="A180" s="1" t="n">
         <v>36494</v>
       </c>
       <c r="B180" t="inlineStr"/>
@@ -4647,7 +4633,7 @@
       <c r="K180" t="inlineStr"/>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n">
+      <c r="A181" s="1" t="n">
         <v>36525</v>
       </c>
       <c r="B181" t="n">
@@ -4680,7 +4666,7 @@
       <c r="K181" t="inlineStr"/>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n">
+      <c r="A182" s="1" t="n">
         <v>36556</v>
       </c>
       <c r="B182" t="inlineStr"/>
@@ -4711,7 +4697,7 @@
       <c r="K182" t="inlineStr"/>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n">
+      <c r="A183" s="1" t="n">
         <v>36585</v>
       </c>
       <c r="B183" t="inlineStr"/>
@@ -4742,7 +4728,7 @@
       <c r="K183" t="inlineStr"/>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n">
+      <c r="A184" s="1" t="n">
         <v>36616</v>
       </c>
       <c r="B184" t="n">
@@ -4775,7 +4761,7 @@
       <c r="K184" t="inlineStr"/>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n">
+      <c r="A185" s="1" t="n">
         <v>36646</v>
       </c>
       <c r="B185" t="inlineStr"/>
@@ -4806,7 +4792,7 @@
       <c r="K185" t="inlineStr"/>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n">
+      <c r="A186" s="1" t="n">
         <v>36677</v>
       </c>
       <c r="B186" t="inlineStr"/>
@@ -4837,7 +4823,7 @@
       <c r="K186" t="inlineStr"/>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n">
+      <c r="A187" s="1" t="n">
         <v>36707</v>
       </c>
       <c r="B187" t="n">
@@ -4870,7 +4856,7 @@
       <c r="K187" t="inlineStr"/>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n">
+      <c r="A188" s="1" t="n">
         <v>36738</v>
       </c>
       <c r="B188" t="inlineStr"/>
@@ -4901,7 +4887,7 @@
       <c r="K188" t="inlineStr"/>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n">
+      <c r="A189" s="1" t="n">
         <v>36769</v>
       </c>
       <c r="B189" t="inlineStr"/>
@@ -4932,7 +4918,7 @@
       <c r="K189" t="inlineStr"/>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n">
+      <c r="A190" s="1" t="n">
         <v>36799</v>
       </c>
       <c r="B190" t="n">
@@ -4965,7 +4951,7 @@
       <c r="K190" t="inlineStr"/>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n">
+      <c r="A191" s="1" t="n">
         <v>36830</v>
       </c>
       <c r="B191" t="inlineStr"/>
@@ -4996,7 +4982,7 @@
       <c r="K191" t="inlineStr"/>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n">
+      <c r="A192" s="1" t="n">
         <v>36860</v>
       </c>
       <c r="B192" t="inlineStr"/>
@@ -5027,7 +5013,7 @@
       <c r="K192" t="inlineStr"/>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n">
+      <c r="A193" s="1" t="n">
         <v>36891</v>
       </c>
       <c r="B193" t="n">
@@ -5060,7 +5046,7 @@
       <c r="K193" t="inlineStr"/>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n">
+      <c r="A194" s="1" t="n">
         <v>36922</v>
       </c>
       <c r="B194" t="inlineStr"/>
@@ -5091,7 +5077,7 @@
       <c r="K194" t="inlineStr"/>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n">
+      <c r="A195" s="1" t="n">
         <v>36950</v>
       </c>
       <c r="B195" t="inlineStr"/>
@@ -5122,7 +5108,7 @@
       <c r="K195" t="inlineStr"/>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n">
+      <c r="A196" s="1" t="n">
         <v>36981</v>
       </c>
       <c r="B196" t="n">
@@ -5155,7 +5141,7 @@
       <c r="K196" t="inlineStr"/>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n">
+      <c r="A197" s="1" t="n">
         <v>37011</v>
       </c>
       <c r="B197" t="inlineStr"/>
@@ -5186,7 +5172,7 @@
       <c r="K197" t="inlineStr"/>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n">
+      <c r="A198" s="1" t="n">
         <v>37042</v>
       </c>
       <c r="B198" t="inlineStr"/>
@@ -5217,7 +5203,7 @@
       <c r="K198" t="inlineStr"/>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n">
+      <c r="A199" s="1" t="n">
         <v>37072</v>
       </c>
       <c r="B199" t="n">
@@ -5250,7 +5236,7 @@
       <c r="K199" t="inlineStr"/>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n">
+      <c r="A200" s="1" t="n">
         <v>37103</v>
       </c>
       <c r="B200" t="inlineStr"/>
@@ -5281,7 +5267,7 @@
       <c r="K200" t="inlineStr"/>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n">
+      <c r="A201" s="1" t="n">
         <v>37134</v>
       </c>
       <c r="B201" t="inlineStr"/>
@@ -5312,7 +5298,7 @@
       <c r="K201" t="inlineStr"/>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n">
+      <c r="A202" s="1" t="n">
         <v>37164</v>
       </c>
       <c r="B202" t="n">
@@ -5345,7 +5331,7 @@
       <c r="K202" t="inlineStr"/>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="n">
+      <c r="A203" s="1" t="n">
         <v>37195</v>
       </c>
       <c r="B203" t="inlineStr"/>
@@ -5376,7 +5362,7 @@
       <c r="K203" t="inlineStr"/>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="n">
+      <c r="A204" s="1" t="n">
         <v>37225</v>
       </c>
       <c r="B204" t="inlineStr"/>
@@ -5407,7 +5393,7 @@
       <c r="K204" t="inlineStr"/>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="n">
+      <c r="A205" s="1" t="n">
         <v>37256</v>
       </c>
       <c r="B205" t="n">
@@ -5440,7 +5426,7 @@
       <c r="K205" t="inlineStr"/>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="n">
+      <c r="A206" s="1" t="n">
         <v>37287</v>
       </c>
       <c r="B206" t="inlineStr"/>
@@ -5471,7 +5457,7 @@
       <c r="K206" t="inlineStr"/>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n">
+      <c r="A207" s="1" t="n">
         <v>37315</v>
       </c>
       <c r="B207" t="inlineStr"/>
@@ -5502,7 +5488,7 @@
       <c r="K207" t="inlineStr"/>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="n">
+      <c r="A208" s="1" t="n">
         <v>37346</v>
       </c>
       <c r="B208" t="n">
@@ -5535,7 +5521,7 @@
       <c r="K208" t="inlineStr"/>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="n">
+      <c r="A209" s="1" t="n">
         <v>37376</v>
       </c>
       <c r="B209" t="inlineStr"/>
@@ -5566,7 +5552,7 @@
       <c r="K209" t="inlineStr"/>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n">
+      <c r="A210" s="1" t="n">
         <v>37407</v>
       </c>
       <c r="B210" t="inlineStr"/>
@@ -5597,7 +5583,7 @@
       <c r="K210" t="inlineStr"/>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="n">
+      <c r="A211" s="1" t="n">
         <v>37437</v>
       </c>
       <c r="B211" t="n">
@@ -5630,7 +5616,7 @@
       <c r="K211" t="inlineStr"/>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="n">
+      <c r="A212" s="1" t="n">
         <v>37468</v>
       </c>
       <c r="B212" t="inlineStr"/>
@@ -5661,7 +5647,7 @@
       <c r="K212" t="inlineStr"/>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="n">
+      <c r="A213" s="1" t="n">
         <v>37499</v>
       </c>
       <c r="B213" t="inlineStr"/>
@@ -5692,7 +5678,7 @@
       <c r="K213" t="inlineStr"/>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="n">
+      <c r="A214" s="1" t="n">
         <v>37529</v>
       </c>
       <c r="B214" t="n">
@@ -5725,7 +5711,7 @@
       <c r="K214" t="inlineStr"/>
     </row>
     <row r="215">
-      <c r="A215" s="2" t="n">
+      <c r="A215" s="1" t="n">
         <v>37560</v>
       </c>
       <c r="B215" t="inlineStr"/>
@@ -5756,7 +5742,7 @@
       <c r="K215" t="inlineStr"/>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="n">
+      <c r="A216" s="1" t="n">
         <v>37590</v>
       </c>
       <c r="B216" t="inlineStr"/>
@@ -5787,7 +5773,7 @@
       <c r="K216" t="inlineStr"/>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="n">
+      <c r="A217" s="1" t="n">
         <v>37621</v>
       </c>
       <c r="B217" t="n">
@@ -5820,7 +5806,7 @@
       <c r="K217" t="inlineStr"/>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="n">
+      <c r="A218" s="1" t="n">
         <v>37652</v>
       </c>
       <c r="B218" t="inlineStr"/>
@@ -5851,7 +5837,7 @@
       <c r="K218" t="inlineStr"/>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="n">
+      <c r="A219" s="1" t="n">
         <v>37680</v>
       </c>
       <c r="B219" t="inlineStr"/>
@@ -5882,7 +5868,7 @@
       <c r="K219" t="inlineStr"/>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n">
+      <c r="A220" s="1" t="n">
         <v>37711</v>
       </c>
       <c r="B220" t="n">
@@ -5915,7 +5901,7 @@
       <c r="K220" t="inlineStr"/>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n">
+      <c r="A221" s="1" t="n">
         <v>37741</v>
       </c>
       <c r="B221" t="inlineStr"/>
@@ -5946,7 +5932,7 @@
       <c r="K221" t="inlineStr"/>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n">
+      <c r="A222" s="1" t="n">
         <v>37772</v>
       </c>
       <c r="B222" t="inlineStr"/>
@@ -5977,7 +5963,7 @@
       <c r="K222" t="inlineStr"/>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n">
+      <c r="A223" s="1" t="n">
         <v>37802</v>
       </c>
       <c r="B223" t="n">
@@ -6010,7 +5996,7 @@
       <c r="K223" t="inlineStr"/>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n">
+      <c r="A224" s="1" t="n">
         <v>37833</v>
       </c>
       <c r="B224" t="inlineStr"/>
@@ -6041,7 +6027,7 @@
       <c r="K224" t="inlineStr"/>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n">
+      <c r="A225" s="1" t="n">
         <v>37864</v>
       </c>
       <c r="B225" t="inlineStr"/>
@@ -6072,7 +6058,7 @@
       <c r="K225" t="inlineStr"/>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n">
+      <c r="A226" s="1" t="n">
         <v>37894</v>
       </c>
       <c r="B226" t="n">
@@ -6105,7 +6091,7 @@
       <c r="K226" t="inlineStr"/>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n">
+      <c r="A227" s="1" t="n">
         <v>37925</v>
       </c>
       <c r="B227" t="inlineStr"/>
@@ -6136,7 +6122,7 @@
       <c r="K227" t="inlineStr"/>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n">
+      <c r="A228" s="1" t="n">
         <v>37955</v>
       </c>
       <c r="B228" t="inlineStr"/>
@@ -6167,7 +6153,7 @@
       <c r="K228" t="inlineStr"/>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n">
+      <c r="A229" s="1" t="n">
         <v>37986</v>
       </c>
       <c r="B229" t="n">
@@ -6200,7 +6186,7 @@
       <c r="K229" t="inlineStr"/>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n">
+      <c r="A230" s="1" t="n">
         <v>38017</v>
       </c>
       <c r="B230" t="inlineStr"/>
@@ -6231,7 +6217,7 @@
       <c r="K230" t="inlineStr"/>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n">
+      <c r="A231" s="1" t="n">
         <v>38046</v>
       </c>
       <c r="B231" t="inlineStr"/>
@@ -6262,7 +6248,7 @@
       <c r="K231" t="inlineStr"/>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n">
+      <c r="A232" s="1" t="n">
         <v>38077</v>
       </c>
       <c r="B232" t="n">
@@ -6295,7 +6281,7 @@
       <c r="K232" t="inlineStr"/>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n">
+      <c r="A233" s="1" t="n">
         <v>38107</v>
       </c>
       <c r="B233" t="inlineStr"/>
@@ -6326,7 +6312,7 @@
       <c r="K233" t="inlineStr"/>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="n">
+      <c r="A234" s="1" t="n">
         <v>38138</v>
       </c>
       <c r="B234" t="inlineStr"/>
@@ -6357,7 +6343,7 @@
       <c r="K234" t="inlineStr"/>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n">
+      <c r="A235" s="1" t="n">
         <v>38168</v>
       </c>
       <c r="B235" t="n">
@@ -6390,7 +6376,7 @@
       <c r="K235" t="inlineStr"/>
     </row>
     <row r="236">
-      <c r="A236" s="2" t="n">
+      <c r="A236" s="1" t="n">
         <v>38199</v>
       </c>
       <c r="B236" t="inlineStr"/>
@@ -6421,7 +6407,7 @@
       <c r="K236" t="inlineStr"/>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="n">
+      <c r="A237" s="1" t="n">
         <v>38230</v>
       </c>
       <c r="B237" t="inlineStr"/>
@@ -6452,7 +6438,7 @@
       <c r="K237" t="inlineStr"/>
     </row>
     <row r="238">
-      <c r="A238" s="2" t="n">
+      <c r="A238" s="1" t="n">
         <v>38260</v>
       </c>
       <c r="B238" t="n">
@@ -6485,7 +6471,7 @@
       <c r="K238" t="inlineStr"/>
     </row>
     <row r="239">
-      <c r="A239" s="2" t="n">
+      <c r="A239" s="1" t="n">
         <v>38291</v>
       </c>
       <c r="B239" t="inlineStr"/>
@@ -6516,7 +6502,7 @@
       <c r="K239" t="inlineStr"/>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="n">
+      <c r="A240" s="1" t="n">
         <v>38321</v>
       </c>
       <c r="B240" t="inlineStr"/>
@@ -6547,7 +6533,7 @@
       <c r="K240" t="inlineStr"/>
     </row>
     <row r="241">
-      <c r="A241" s="2" t="n">
+      <c r="A241" s="1" t="n">
         <v>38352</v>
       </c>
       <c r="B241" t="n">
@@ -6580,7 +6566,7 @@
       <c r="K241" t="inlineStr"/>
     </row>
     <row r="242">
-      <c r="A242" s="2" t="n">
+      <c r="A242" s="1" t="n">
         <v>38383</v>
       </c>
       <c r="B242" t="inlineStr"/>
@@ -6611,7 +6597,7 @@
       <c r="K242" t="inlineStr"/>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="n">
+      <c r="A243" s="1" t="n">
         <v>38411</v>
       </c>
       <c r="B243" t="inlineStr"/>
@@ -6642,7 +6628,7 @@
       <c r="K243" t="inlineStr"/>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="n">
+      <c r="A244" s="1" t="n">
         <v>38442</v>
       </c>
       <c r="B244" t="n">
@@ -6675,7 +6661,7 @@
       <c r="K244" t="inlineStr"/>
     </row>
     <row r="245">
-      <c r="A245" s="2" t="n">
+      <c r="A245" s="1" t="n">
         <v>38472</v>
       </c>
       <c r="B245" t="inlineStr"/>
@@ -6706,7 +6692,7 @@
       <c r="K245" t="inlineStr"/>
     </row>
     <row r="246">
-      <c r="A246" s="2" t="n">
+      <c r="A246" s="1" t="n">
         <v>38503</v>
       </c>
       <c r="B246" t="inlineStr"/>
@@ -6737,7 +6723,7 @@
       <c r="K246" t="inlineStr"/>
     </row>
     <row r="247">
-      <c r="A247" s="2" t="n">
+      <c r="A247" s="1" t="n">
         <v>38533</v>
       </c>
       <c r="B247" t="n">
@@ -6770,7 +6756,7 @@
       <c r="K247" t="inlineStr"/>
     </row>
     <row r="248">
-      <c r="A248" s="2" t="n">
+      <c r="A248" s="1" t="n">
         <v>38564</v>
       </c>
       <c r="B248" t="inlineStr"/>
@@ -6801,7 +6787,7 @@
       <c r="K248" t="inlineStr"/>
     </row>
     <row r="249">
-      <c r="A249" s="2" t="n">
+      <c r="A249" s="1" t="n">
         <v>38595</v>
       </c>
       <c r="B249" t="inlineStr"/>
@@ -6832,7 +6818,7 @@
       <c r="K249" t="inlineStr"/>
     </row>
     <row r="250">
-      <c r="A250" s="2" t="n">
+      <c r="A250" s="1" t="n">
         <v>38625</v>
       </c>
       <c r="B250" t="n">
@@ -6865,7 +6851,7 @@
       <c r="K250" t="inlineStr"/>
     </row>
     <row r="251">
-      <c r="A251" s="2" t="n">
+      <c r="A251" s="1" t="n">
         <v>38656</v>
       </c>
       <c r="B251" t="inlineStr"/>
@@ -6896,7 +6882,7 @@
       <c r="K251" t="inlineStr"/>
     </row>
     <row r="252">
-      <c r="A252" s="2" t="n">
+      <c r="A252" s="1" t="n">
         <v>38686</v>
       </c>
       <c r="B252" t="inlineStr"/>
@@ -6927,7 +6913,7 @@
       <c r="K252" t="inlineStr"/>
     </row>
     <row r="253">
-      <c r="A253" s="2" t="n">
+      <c r="A253" s="1" t="n">
         <v>38717</v>
       </c>
       <c r="B253" t="n">
@@ -6960,7 +6946,7 @@
       <c r="K253" t="inlineStr"/>
     </row>
     <row r="254">
-      <c r="A254" s="2" t="n">
+      <c r="A254" s="1" t="n">
         <v>38748</v>
       </c>
       <c r="B254" t="inlineStr"/>
@@ -6991,7 +6977,7 @@
       <c r="K254" t="inlineStr"/>
     </row>
     <row r="255">
-      <c r="A255" s="2" t="n">
+      <c r="A255" s="1" t="n">
         <v>38776</v>
       </c>
       <c r="B255" t="inlineStr"/>
@@ -7022,7 +7008,7 @@
       <c r="K255" t="inlineStr"/>
     </row>
     <row r="256">
-      <c r="A256" s="2" t="n">
+      <c r="A256" s="1" t="n">
         <v>38807</v>
       </c>
       <c r="B256" t="n">
@@ -7055,7 +7041,7 @@
       <c r="K256" t="inlineStr"/>
     </row>
     <row r="257">
-      <c r="A257" s="2" t="n">
+      <c r="A257" s="1" t="n">
         <v>38837</v>
       </c>
       <c r="B257" t="inlineStr"/>
@@ -7086,7 +7072,7 @@
       <c r="K257" t="inlineStr"/>
     </row>
     <row r="258">
-      <c r="A258" s="2" t="n">
+      <c r="A258" s="1" t="n">
         <v>38868</v>
       </c>
       <c r="B258" t="inlineStr"/>
@@ -7117,7 +7103,7 @@
       <c r="K258" t="inlineStr"/>
     </row>
     <row r="259">
-      <c r="A259" s="2" t="n">
+      <c r="A259" s="1" t="n">
         <v>38898</v>
       </c>
       <c r="B259" t="n">
@@ -7150,7 +7136,7 @@
       <c r="K259" t="inlineStr"/>
     </row>
     <row r="260">
-      <c r="A260" s="2" t="n">
+      <c r="A260" s="1" t="n">
         <v>38929</v>
       </c>
       <c r="B260" t="inlineStr"/>
@@ -7181,7 +7167,7 @@
       <c r="K260" t="inlineStr"/>
     </row>
     <row r="261">
-      <c r="A261" s="2" t="n">
+      <c r="A261" s="1" t="n">
         <v>38960</v>
       </c>
       <c r="B261" t="inlineStr"/>
@@ -7212,7 +7198,7 @@
       <c r="K261" t="inlineStr"/>
     </row>
     <row r="262">
-      <c r="A262" s="2" t="n">
+      <c r="A262" s="1" t="n">
         <v>38990</v>
       </c>
       <c r="B262" t="n">
@@ -7245,7 +7231,7 @@
       <c r="K262" t="inlineStr"/>
     </row>
     <row r="263">
-      <c r="A263" s="2" t="n">
+      <c r="A263" s="1" t="n">
         <v>39021</v>
       </c>
       <c r="B263" t="inlineStr"/>
@@ -7276,7 +7262,7 @@
       <c r="K263" t="inlineStr"/>
     </row>
     <row r="264">
-      <c r="A264" s="2" t="n">
+      <c r="A264" s="1" t="n">
         <v>39051</v>
       </c>
       <c r="B264" t="inlineStr"/>
@@ -7307,7 +7293,7 @@
       <c r="K264" t="inlineStr"/>
     </row>
     <row r="265">
-      <c r="A265" s="2" t="n">
+      <c r="A265" s="1" t="n">
         <v>39082</v>
       </c>
       <c r="B265" t="n">
@@ -7340,7 +7326,7 @@
       <c r="K265" t="inlineStr"/>
     </row>
     <row r="266">
-      <c r="A266" s="2" t="n">
+      <c r="A266" s="1" t="n">
         <v>39113</v>
       </c>
       <c r="B266" t="inlineStr"/>
@@ -7371,7 +7357,7 @@
       <c r="K266" t="inlineStr"/>
     </row>
     <row r="267">
-      <c r="A267" s="2" t="n">
+      <c r="A267" s="1" t="n">
         <v>39141</v>
       </c>
       <c r="B267" t="inlineStr"/>
@@ -7402,7 +7388,7 @@
       <c r="K267" t="inlineStr"/>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="n">
+      <c r="A268" s="1" t="n">
         <v>39172</v>
       </c>
       <c r="B268" t="n">
@@ -7435,7 +7421,7 @@
       <c r="K268" t="inlineStr"/>
     </row>
     <row r="269">
-      <c r="A269" s="2" t="n">
+      <c r="A269" s="1" t="n">
         <v>39202</v>
       </c>
       <c r="B269" t="inlineStr"/>
@@ -7466,7 +7452,7 @@
       <c r="K269" t="inlineStr"/>
     </row>
     <row r="270">
-      <c r="A270" s="2" t="n">
+      <c r="A270" s="1" t="n">
         <v>39233</v>
       </c>
       <c r="B270" t="inlineStr"/>
@@ -7497,7 +7483,7 @@
       <c r="K270" t="inlineStr"/>
     </row>
     <row r="271">
-      <c r="A271" s="2" t="n">
+      <c r="A271" s="1" t="n">
         <v>39263</v>
       </c>
       <c r="B271" t="n">
@@ -7530,7 +7516,7 @@
       <c r="K271" t="inlineStr"/>
     </row>
     <row r="272">
-      <c r="A272" s="2" t="n">
+      <c r="A272" s="1" t="n">
         <v>39294</v>
       </c>
       <c r="B272" t="inlineStr"/>
@@ -7561,7 +7547,7 @@
       <c r="K272" t="inlineStr"/>
     </row>
     <row r="273">
-      <c r="A273" s="2" t="n">
+      <c r="A273" s="1" t="n">
         <v>39325</v>
       </c>
       <c r="B273" t="inlineStr"/>
@@ -7592,7 +7578,7 @@
       <c r="K273" t="inlineStr"/>
     </row>
     <row r="274">
-      <c r="A274" s="2" t="n">
+      <c r="A274" s="1" t="n">
         <v>39355</v>
       </c>
       <c r="B274" t="n">
@@ -7625,7 +7611,7 @@
       <c r="K274" t="inlineStr"/>
     </row>
     <row r="275">
-      <c r="A275" s="2" t="n">
+      <c r="A275" s="1" t="n">
         <v>39386</v>
       </c>
       <c r="B275" t="inlineStr"/>
@@ -7656,7 +7642,7 @@
       <c r="K275" t="inlineStr"/>
     </row>
     <row r="276">
-      <c r="A276" s="2" t="n">
+      <c r="A276" s="1" t="n">
         <v>39416</v>
       </c>
       <c r="B276" t="inlineStr"/>
@@ -7687,7 +7673,7 @@
       <c r="K276" t="inlineStr"/>
     </row>
     <row r="277">
-      <c r="A277" s="2" t="n">
+      <c r="A277" s="1" t="n">
         <v>39447</v>
       </c>
       <c r="B277" t="n">
@@ -7720,7 +7706,7 @@
       <c r="K277" t="inlineStr"/>
     </row>
     <row r="278">
-      <c r="A278" s="2" t="n">
+      <c r="A278" s="1" t="n">
         <v>39478</v>
       </c>
       <c r="B278" t="inlineStr"/>
@@ -7751,7 +7737,7 @@
       <c r="K278" t="inlineStr"/>
     </row>
     <row r="279">
-      <c r="A279" s="2" t="n">
+      <c r="A279" s="1" t="n">
         <v>39507</v>
       </c>
       <c r="B279" t="inlineStr"/>
@@ -7782,7 +7768,7 @@
       <c r="K279" t="inlineStr"/>
     </row>
     <row r="280">
-      <c r="A280" s="2" t="n">
+      <c r="A280" s="1" t="n">
         <v>39538</v>
       </c>
       <c r="B280" t="n">
@@ -7815,7 +7801,7 @@
       <c r="K280" t="inlineStr"/>
     </row>
     <row r="281">
-      <c r="A281" s="2" t="n">
+      <c r="A281" s="1" t="n">
         <v>39568</v>
       </c>
       <c r="B281" t="inlineStr"/>
@@ -7846,7 +7832,7 @@
       <c r="K281" t="inlineStr"/>
     </row>
     <row r="282">
-      <c r="A282" s="2" t="n">
+      <c r="A282" s="1" t="n">
         <v>39599</v>
       </c>
       <c r="B282" t="inlineStr"/>
@@ -7877,7 +7863,7 @@
       <c r="K282" t="inlineStr"/>
     </row>
     <row r="283">
-      <c r="A283" s="2" t="n">
+      <c r="A283" s="1" t="n">
         <v>39629</v>
       </c>
       <c r="B283" t="n">
@@ -7910,7 +7896,7 @@
       <c r="K283" t="inlineStr"/>
     </row>
     <row r="284">
-      <c r="A284" s="2" t="n">
+      <c r="A284" s="1" t="n">
         <v>39660</v>
       </c>
       <c r="B284" t="inlineStr"/>
@@ -7941,7 +7927,7 @@
       <c r="K284" t="inlineStr"/>
     </row>
     <row r="285">
-      <c r="A285" s="2" t="n">
+      <c r="A285" s="1" t="n">
         <v>39691</v>
       </c>
       <c r="B285" t="inlineStr"/>
@@ -7972,7 +7958,7 @@
       <c r="K285" t="inlineStr"/>
     </row>
     <row r="286">
-      <c r="A286" s="2" t="n">
+      <c r="A286" s="1" t="n">
         <v>39721</v>
       </c>
       <c r="B286" t="n">
@@ -8005,7 +7991,7 @@
       <c r="K286" t="inlineStr"/>
     </row>
     <row r="287">
-      <c r="A287" s="2" t="n">
+      <c r="A287" s="1" t="n">
         <v>39752</v>
       </c>
       <c r="B287" t="inlineStr"/>
@@ -8036,7 +8022,7 @@
       <c r="K287" t="inlineStr"/>
     </row>
     <row r="288">
-      <c r="A288" s="2" t="n">
+      <c r="A288" s="1" t="n">
         <v>39782</v>
       </c>
       <c r="B288" t="inlineStr"/>
@@ -8067,7 +8053,7 @@
       <c r="K288" t="inlineStr"/>
     </row>
     <row r="289">
-      <c r="A289" s="2" t="n">
+      <c r="A289" s="1" t="n">
         <v>39813</v>
       </c>
       <c r="B289" t="n">
@@ -8100,7 +8086,7 @@
       <c r="K289" t="inlineStr"/>
     </row>
     <row r="290">
-      <c r="A290" s="2" t="n">
+      <c r="A290" s="1" t="n">
         <v>39844</v>
       </c>
       <c r="B290" t="inlineStr"/>
@@ -8131,7 +8117,7 @@
       <c r="K290" t="inlineStr"/>
     </row>
     <row r="291">
-      <c r="A291" s="2" t="n">
+      <c r="A291" s="1" t="n">
         <v>39872</v>
       </c>
       <c r="B291" t="inlineStr"/>
@@ -8162,7 +8148,7 @@
       <c r="K291" t="inlineStr"/>
     </row>
     <row r="292">
-      <c r="A292" s="2" t="n">
+      <c r="A292" s="1" t="n">
         <v>39903</v>
       </c>
       <c r="B292" t="n">
@@ -8195,7 +8181,7 @@
       <c r="K292" t="inlineStr"/>
     </row>
     <row r="293">
-      <c r="A293" s="2" t="n">
+      <c r="A293" s="1" t="n">
         <v>39933</v>
       </c>
       <c r="B293" t="inlineStr"/>
@@ -8226,7 +8212,7 @@
       <c r="K293" t="inlineStr"/>
     </row>
     <row r="294">
-      <c r="A294" s="2" t="n">
+      <c r="A294" s="1" t="n">
         <v>39964</v>
       </c>
       <c r="B294" t="inlineStr"/>
@@ -8257,7 +8243,7 @@
       <c r="K294" t="inlineStr"/>
     </row>
     <row r="295">
-      <c r="A295" s="2" t="n">
+      <c r="A295" s="1" t="n">
         <v>39994</v>
       </c>
       <c r="B295" t="n">
@@ -8290,7 +8276,7 @@
       <c r="K295" t="inlineStr"/>
     </row>
     <row r="296">
-      <c r="A296" s="2" t="n">
+      <c r="A296" s="1" t="n">
         <v>40025</v>
       </c>
       <c r="B296" t="inlineStr"/>
@@ -8321,7 +8307,7 @@
       <c r="K296" t="inlineStr"/>
     </row>
     <row r="297">
-      <c r="A297" s="2" t="n">
+      <c r="A297" s="1" t="n">
         <v>40056</v>
       </c>
       <c r="B297" t="inlineStr"/>
@@ -8352,7 +8338,7 @@
       <c r="K297" t="inlineStr"/>
     </row>
     <row r="298">
-      <c r="A298" s="2" t="n">
+      <c r="A298" s="1" t="n">
         <v>40086</v>
       </c>
       <c r="B298" t="n">
@@ -8385,7 +8371,7 @@
       <c r="K298" t="inlineStr"/>
     </row>
     <row r="299">
-      <c r="A299" s="2" t="n">
+      <c r="A299" s="1" t="n">
         <v>40117</v>
       </c>
       <c r="B299" t="inlineStr"/>
@@ -8416,7 +8402,7 @@
       <c r="K299" t="inlineStr"/>
     </row>
     <row r="300">
-      <c r="A300" s="2" t="n">
+      <c r="A300" s="1" t="n">
         <v>40147</v>
       </c>
       <c r="B300" t="inlineStr"/>
@@ -8447,7 +8433,7 @@
       <c r="K300" t="inlineStr"/>
     </row>
     <row r="301">
-      <c r="A301" s="2" t="n">
+      <c r="A301" s="1" t="n">
         <v>40178</v>
       </c>
       <c r="B301" t="n">
@@ -8480,7 +8466,7 @@
       <c r="K301" t="inlineStr"/>
     </row>
     <row r="302">
-      <c r="A302" s="2" t="n">
+      <c r="A302" s="1" t="n">
         <v>40209</v>
       </c>
       <c r="B302" t="inlineStr"/>
@@ -8511,7 +8497,7 @@
       <c r="K302" t="inlineStr"/>
     </row>
     <row r="303">
-      <c r="A303" s="2" t="n">
+      <c r="A303" s="1" t="n">
         <v>40237</v>
       </c>
       <c r="B303" t="inlineStr"/>
@@ -8542,7 +8528,7 @@
       <c r="K303" t="inlineStr"/>
     </row>
     <row r="304">
-      <c r="A304" s="2" t="n">
+      <c r="A304" s="1" t="n">
         <v>40268</v>
       </c>
       <c r="B304" t="n">
@@ -8575,7 +8561,7 @@
       <c r="K304" t="inlineStr"/>
     </row>
     <row r="305">
-      <c r="A305" s="2" t="n">
+      <c r="A305" s="1" t="n">
         <v>40298</v>
       </c>
       <c r="B305" t="inlineStr"/>
@@ -8606,7 +8592,7 @@
       <c r="K305" t="inlineStr"/>
     </row>
     <row r="306">
-      <c r="A306" s="2" t="n">
+      <c r="A306" s="1" t="n">
         <v>40329</v>
       </c>
       <c r="B306" t="inlineStr"/>
@@ -8637,7 +8623,7 @@
       <c r="K306" t="inlineStr"/>
     </row>
     <row r="307">
-      <c r="A307" s="2" t="n">
+      <c r="A307" s="1" t="n">
         <v>40359</v>
       </c>
       <c r="B307" t="n">
@@ -8670,7 +8656,7 @@
       <c r="K307" t="inlineStr"/>
     </row>
     <row r="308">
-      <c r="A308" s="2" t="n">
+      <c r="A308" s="1" t="n">
         <v>40390</v>
       </c>
       <c r="B308" t="inlineStr"/>
@@ -8701,7 +8687,7 @@
       <c r="K308" t="inlineStr"/>
     </row>
     <row r="309">
-      <c r="A309" s="2" t="n">
+      <c r="A309" s="1" t="n">
         <v>40421</v>
       </c>
       <c r="B309" t="inlineStr"/>
@@ -8732,7 +8718,7 @@
       <c r="K309" t="inlineStr"/>
     </row>
     <row r="310">
-      <c r="A310" s="2" t="n">
+      <c r="A310" s="1" t="n">
         <v>40451</v>
       </c>
       <c r="B310" t="n">
@@ -8765,7 +8751,7 @@
       <c r="K310" t="inlineStr"/>
     </row>
     <row r="311">
-      <c r="A311" s="2" t="n">
+      <c r="A311" s="1" t="n">
         <v>40482</v>
       </c>
       <c r="B311" t="inlineStr"/>
@@ -8796,7 +8782,7 @@
       <c r="K311" t="inlineStr"/>
     </row>
     <row r="312">
-      <c r="A312" s="2" t="n">
+      <c r="A312" s="1" t="n">
         <v>40512</v>
       </c>
       <c r="B312" t="inlineStr"/>
@@ -8827,7 +8813,7 @@
       <c r="K312" t="inlineStr"/>
     </row>
     <row r="313">
-      <c r="A313" s="2" t="n">
+      <c r="A313" s="1" t="n">
         <v>40543</v>
       </c>
       <c r="B313" t="n">
@@ -8860,7 +8846,7 @@
       <c r="K313" t="inlineStr"/>
     </row>
     <row r="314">
-      <c r="A314" s="2" t="n">
+      <c r="A314" s="1" t="n">
         <v>40574</v>
       </c>
       <c r="B314" t="inlineStr"/>
@@ -8891,7 +8877,7 @@
       <c r="K314" t="inlineStr"/>
     </row>
     <row r="315">
-      <c r="A315" s="2" t="n">
+      <c r="A315" s="1" t="n">
         <v>40602</v>
       </c>
       <c r="B315" t="inlineStr"/>
@@ -8922,7 +8908,7 @@
       <c r="K315" t="inlineStr"/>
     </row>
     <row r="316">
-      <c r="A316" s="2" t="n">
+      <c r="A316" s="1" t="n">
         <v>40633</v>
       </c>
       <c r="B316" t="n">
@@ -8955,7 +8941,7 @@
       <c r="K316" t="inlineStr"/>
     </row>
     <row r="317">
-      <c r="A317" s="2" t="n">
+      <c r="A317" s="1" t="n">
         <v>40663</v>
       </c>
       <c r="B317" t="inlineStr"/>
@@ -8986,7 +8972,7 @@
       <c r="K317" t="inlineStr"/>
     </row>
     <row r="318">
-      <c r="A318" s="2" t="n">
+      <c r="A318" s="1" t="n">
         <v>40694</v>
       </c>
       <c r="B318" t="inlineStr"/>
@@ -9017,7 +9003,7 @@
       <c r="K318" t="inlineStr"/>
     </row>
     <row r="319">
-      <c r="A319" s="2" t="n">
+      <c r="A319" s="1" t="n">
         <v>40724</v>
       </c>
       <c r="B319" t="n">
@@ -9050,7 +9036,7 @@
       <c r="K319" t="inlineStr"/>
     </row>
     <row r="320">
-      <c r="A320" s="2" t="n">
+      <c r="A320" s="1" t="n">
         <v>40755</v>
       </c>
       <c r="B320" t="inlineStr"/>
@@ -9081,7 +9067,7 @@
       <c r="K320" t="inlineStr"/>
     </row>
     <row r="321">
-      <c r="A321" s="2" t="n">
+      <c r="A321" s="1" t="n">
         <v>40786</v>
       </c>
       <c r="B321" t="inlineStr"/>
@@ -9112,7 +9098,7 @@
       <c r="K321" t="inlineStr"/>
     </row>
     <row r="322">
-      <c r="A322" s="2" t="n">
+      <c r="A322" s="1" t="n">
         <v>40816</v>
       </c>
       <c r="B322" t="n">
@@ -9145,7 +9131,7 @@
       <c r="K322" t="inlineStr"/>
     </row>
     <row r="323">
-      <c r="A323" s="2" t="n">
+      <c r="A323" s="1" t="n">
         <v>40847</v>
       </c>
       <c r="B323" t="inlineStr"/>
@@ -9176,7 +9162,7 @@
       <c r="K323" t="inlineStr"/>
     </row>
     <row r="324">
-      <c r="A324" s="2" t="n">
+      <c r="A324" s="1" t="n">
         <v>40877</v>
       </c>
       <c r="B324" t="inlineStr"/>
@@ -9207,7 +9193,7 @@
       <c r="K324" t="inlineStr"/>
     </row>
     <row r="325">
-      <c r="A325" s="2" t="n">
+      <c r="A325" s="1" t="n">
         <v>40908</v>
       </c>
       <c r="B325" t="n">
@@ -9240,7 +9226,7 @@
       <c r="K325" t="inlineStr"/>
     </row>
     <row r="326">
-      <c r="A326" s="2" t="n">
+      <c r="A326" s="1" t="n">
         <v>40939</v>
       </c>
       <c r="B326" t="inlineStr"/>
@@ -9271,7 +9257,7 @@
       <c r="K326" t="inlineStr"/>
     </row>
     <row r="327">
-      <c r="A327" s="2" t="n">
+      <c r="A327" s="1" t="n">
         <v>40968</v>
       </c>
       <c r="B327" t="inlineStr"/>
@@ -9302,7 +9288,7 @@
       <c r="K327" t="inlineStr"/>
     </row>
     <row r="328">
-      <c r="A328" s="2" t="n">
+      <c r="A328" s="1" t="n">
         <v>40999</v>
       </c>
       <c r="B328" t="n">
@@ -9335,7 +9321,7 @@
       <c r="K328" t="inlineStr"/>
     </row>
     <row r="329">
-      <c r="A329" s="2" t="n">
+      <c r="A329" s="1" t="n">
         <v>41029</v>
       </c>
       <c r="B329" t="inlineStr"/>
@@ -9366,7 +9352,7 @@
       <c r="K329" t="inlineStr"/>
     </row>
     <row r="330">
-      <c r="A330" s="2" t="n">
+      <c r="A330" s="1" t="n">
         <v>41060</v>
       </c>
       <c r="B330" t="inlineStr"/>
@@ -9397,7 +9383,7 @@
       <c r="K330" t="inlineStr"/>
     </row>
     <row r="331">
-      <c r="A331" s="2" t="n">
+      <c r="A331" s="1" t="n">
         <v>41090</v>
       </c>
       <c r="B331" t="n">
@@ -9430,7 +9416,7 @@
       <c r="K331" t="inlineStr"/>
     </row>
     <row r="332">
-      <c r="A332" s="2" t="n">
+      <c r="A332" s="1" t="n">
         <v>41121</v>
       </c>
       <c r="B332" t="inlineStr"/>
@@ -9461,7 +9447,7 @@
       <c r="K332" t="inlineStr"/>
     </row>
     <row r="333">
-      <c r="A333" s="2" t="n">
+      <c r="A333" s="1" t="n">
         <v>41152</v>
       </c>
       <c r="B333" t="inlineStr"/>
@@ -9492,7 +9478,7 @@
       <c r="K333" t="inlineStr"/>
     </row>
     <row r="334">
-      <c r="A334" s="2" t="n">
+      <c r="A334" s="1" t="n">
         <v>41182</v>
       </c>
       <c r="B334" t="n">
@@ -9525,7 +9511,7 @@
       <c r="K334" t="inlineStr"/>
     </row>
     <row r="335">
-      <c r="A335" s="2" t="n">
+      <c r="A335" s="1" t="n">
         <v>41213</v>
       </c>
       <c r="B335" t="inlineStr"/>
@@ -9556,7 +9542,7 @@
       <c r="K335" t="inlineStr"/>
     </row>
     <row r="336">
-      <c r="A336" s="2" t="n">
+      <c r="A336" s="1" t="n">
         <v>41243</v>
       </c>
       <c r="B336" t="inlineStr"/>
@@ -9587,7 +9573,7 @@
       <c r="K336" t="inlineStr"/>
     </row>
     <row r="337">
-      <c r="A337" s="2" t="n">
+      <c r="A337" s="1" t="n">
         <v>41274</v>
       </c>
       <c r="B337" t="n">
@@ -9620,7 +9606,7 @@
       <c r="K337" t="inlineStr"/>
     </row>
     <row r="338">
-      <c r="A338" s="2" t="n">
+      <c r="A338" s="1" t="n">
         <v>41305</v>
       </c>
       <c r="B338" t="inlineStr"/>
@@ -9651,7 +9637,7 @@
       <c r="K338" t="inlineStr"/>
     </row>
     <row r="339">
-      <c r="A339" s="2" t="n">
+      <c r="A339" s="1" t="n">
         <v>41333</v>
       </c>
       <c r="B339" t="inlineStr"/>
@@ -9682,7 +9668,7 @@
       <c r="K339" t="inlineStr"/>
     </row>
     <row r="340">
-      <c r="A340" s="2" t="n">
+      <c r="A340" s="1" t="n">
         <v>41364</v>
       </c>
       <c r="B340" t="n">
@@ -9715,7 +9701,7 @@
       <c r="K340" t="inlineStr"/>
     </row>
     <row r="341">
-      <c r="A341" s="2" t="n">
+      <c r="A341" s="1" t="n">
         <v>41394</v>
       </c>
       <c r="B341" t="inlineStr"/>
@@ -9746,7 +9732,7 @@
       <c r="K341" t="inlineStr"/>
     </row>
     <row r="342">
-      <c r="A342" s="2" t="n">
+      <c r="A342" s="1" t="n">
         <v>41425</v>
       </c>
       <c r="B342" t="inlineStr"/>
@@ -9777,7 +9763,7 @@
       <c r="K342" t="inlineStr"/>
     </row>
     <row r="343">
-      <c r="A343" s="2" t="n">
+      <c r="A343" s="1" t="n">
         <v>41455</v>
       </c>
       <c r="B343" t="n">
@@ -9810,7 +9796,7 @@
       <c r="K343" t="inlineStr"/>
     </row>
     <row r="344">
-      <c r="A344" s="2" t="n">
+      <c r="A344" s="1" t="n">
         <v>41486</v>
       </c>
       <c r="B344" t="inlineStr"/>
@@ -9841,7 +9827,7 @@
       <c r="K344" t="inlineStr"/>
     </row>
     <row r="345">
-      <c r="A345" s="2" t="n">
+      <c r="A345" s="1" t="n">
         <v>41517</v>
       </c>
       <c r="B345" t="inlineStr"/>
@@ -9872,7 +9858,7 @@
       <c r="K345" t="inlineStr"/>
     </row>
     <row r="346">
-      <c r="A346" s="2" t="n">
+      <c r="A346" s="1" t="n">
         <v>41547</v>
       </c>
       <c r="B346" t="n">
@@ -9905,7 +9891,7 @@
       <c r="K346" t="inlineStr"/>
     </row>
     <row r="347">
-      <c r="A347" s="2" t="n">
+      <c r="A347" s="1" t="n">
         <v>41578</v>
       </c>
       <c r="B347" t="inlineStr"/>
@@ -9936,7 +9922,7 @@
       <c r="K347" t="inlineStr"/>
     </row>
     <row r="348">
-      <c r="A348" s="2" t="n">
+      <c r="A348" s="1" t="n">
         <v>41608</v>
       </c>
       <c r="B348" t="inlineStr"/>
@@ -9967,7 +9953,7 @@
       <c r="K348" t="inlineStr"/>
     </row>
     <row r="349">
-      <c r="A349" s="2" t="n">
+      <c r="A349" s="1" t="n">
         <v>41639</v>
       </c>
       <c r="B349" t="n">
@@ -10000,7 +9986,7 @@
       <c r="K349" t="inlineStr"/>
     </row>
     <row r="350">
-      <c r="A350" s="2" t="n">
+      <c r="A350" s="1" t="n">
         <v>41670</v>
       </c>
       <c r="B350" t="inlineStr"/>
@@ -10031,7 +10017,7 @@
       <c r="K350" t="inlineStr"/>
     </row>
     <row r="351">
-      <c r="A351" s="2" t="n">
+      <c r="A351" s="1" t="n">
         <v>41698</v>
       </c>
       <c r="B351" t="inlineStr"/>
@@ -10062,7 +10048,7 @@
       <c r="K351" t="inlineStr"/>
     </row>
     <row r="352">
-      <c r="A352" s="2" t="n">
+      <c r="A352" s="1" t="n">
         <v>41729</v>
       </c>
       <c r="B352" t="n">
@@ -10095,7 +10081,7 @@
       <c r="K352" t="inlineStr"/>
     </row>
     <row r="353">
-      <c r="A353" s="2" t="n">
+      <c r="A353" s="1" t="n">
         <v>41759</v>
       </c>
       <c r="B353" t="inlineStr"/>
@@ -10126,7 +10112,7 @@
       <c r="K353" t="inlineStr"/>
     </row>
     <row r="354">
-      <c r="A354" s="2" t="n">
+      <c r="A354" s="1" t="n">
         <v>41790</v>
       </c>
       <c r="B354" t="inlineStr"/>
@@ -10157,7 +10143,7 @@
       <c r="K354" t="inlineStr"/>
     </row>
     <row r="355">
-      <c r="A355" s="2" t="n">
+      <c r="A355" s="1" t="n">
         <v>41820</v>
       </c>
       <c r="B355" t="n">
@@ -10190,7 +10176,7 @@
       <c r="K355" t="inlineStr"/>
     </row>
     <row r="356">
-      <c r="A356" s="2" t="n">
+      <c r="A356" s="1" t="n">
         <v>41851</v>
       </c>
       <c r="B356" t="inlineStr"/>
@@ -10221,7 +10207,7 @@
       <c r="K356" t="inlineStr"/>
     </row>
     <row r="357">
-      <c r="A357" s="2" t="n">
+      <c r="A357" s="1" t="n">
         <v>41882</v>
       </c>
       <c r="B357" t="inlineStr"/>
@@ -10252,7 +10238,7 @@
       <c r="K357" t="inlineStr"/>
     </row>
     <row r="358">
-      <c r="A358" s="2" t="n">
+      <c r="A358" s="1" t="n">
         <v>41912</v>
       </c>
       <c r="B358" t="n">
@@ -10285,7 +10271,7 @@
       <c r="K358" t="inlineStr"/>
     </row>
     <row r="359">
-      <c r="A359" s="2" t="n">
+      <c r="A359" s="1" t="n">
         <v>41943</v>
       </c>
       <c r="B359" t="inlineStr"/>
@@ -10316,7 +10302,7 @@
       <c r="K359" t="inlineStr"/>
     </row>
     <row r="360">
-      <c r="A360" s="2" t="n">
+      <c r="A360" s="1" t="n">
         <v>41973</v>
       </c>
       <c r="B360" t="inlineStr"/>
@@ -10347,7 +10333,7 @@
       <c r="K360" t="inlineStr"/>
     </row>
     <row r="361">
-      <c r="A361" s="2" t="n">
+      <c r="A361" s="1" t="n">
         <v>42004</v>
       </c>
       <c r="B361" t="n">
@@ -10380,7 +10366,7 @@
       <c r="K361" t="inlineStr"/>
     </row>
     <row r="362">
-      <c r="A362" s="2" t="n">
+      <c r="A362" s="1" t="n">
         <v>42035</v>
       </c>
       <c r="B362" t="inlineStr"/>
@@ -10411,7 +10397,7 @@
       <c r="K362" t="inlineStr"/>
     </row>
     <row r="363">
-      <c r="A363" s="2" t="n">
+      <c r="A363" s="1" t="n">
         <v>42063</v>
       </c>
       <c r="B363" t="inlineStr"/>
@@ -10442,7 +10428,7 @@
       <c r="K363" t="inlineStr"/>
     </row>
     <row r="364">
-      <c r="A364" s="2" t="n">
+      <c r="A364" s="1" t="n">
         <v>42094</v>
       </c>
       <c r="B364" t="n">
@@ -10475,7 +10461,7 @@
       <c r="K364" t="inlineStr"/>
     </row>
     <row r="365">
-      <c r="A365" s="2" t="n">
+      <c r="A365" s="1" t="n">
         <v>42124</v>
       </c>
       <c r="B365" t="inlineStr"/>
@@ -10506,7 +10492,7 @@
       <c r="K365" t="inlineStr"/>
     </row>
     <row r="366">
-      <c r="A366" s="2" t="n">
+      <c r="A366" s="1" t="n">
         <v>42155</v>
       </c>
       <c r="B366" t="inlineStr"/>
@@ -10537,7 +10523,7 @@
       <c r="K366" t="inlineStr"/>
     </row>
     <row r="367">
-      <c r="A367" s="2" t="n">
+      <c r="A367" s="1" t="n">
         <v>42185</v>
       </c>
       <c r="B367" t="n">
@@ -10570,7 +10556,7 @@
       <c r="K367" t="inlineStr"/>
     </row>
     <row r="368">
-      <c r="A368" s="2" t="n">
+      <c r="A368" s="1" t="n">
         <v>42216</v>
       </c>
       <c r="B368" t="inlineStr"/>
@@ -10601,7 +10587,7 @@
       <c r="K368" t="inlineStr"/>
     </row>
     <row r="369">
-      <c r="A369" s="2" t="n">
+      <c r="A369" s="1" t="n">
         <v>42247</v>
       </c>
       <c r="B369" t="inlineStr"/>
@@ -10632,7 +10618,7 @@
       <c r="K369" t="inlineStr"/>
     </row>
     <row r="370">
-      <c r="A370" s="2" t="n">
+      <c r="A370" s="1" t="n">
         <v>42277</v>
       </c>
       <c r="B370" t="n">
@@ -10665,7 +10651,7 @@
       <c r="K370" t="inlineStr"/>
     </row>
     <row r="371">
-      <c r="A371" s="2" t="n">
+      <c r="A371" s="1" t="n">
         <v>42308</v>
       </c>
       <c r="B371" t="inlineStr"/>
@@ -10696,7 +10682,7 @@
       <c r="K371" t="inlineStr"/>
     </row>
     <row r="372">
-      <c r="A372" s="2" t="n">
+      <c r="A372" s="1" t="n">
         <v>42338</v>
       </c>
       <c r="B372" t="inlineStr"/>
@@ -10727,7 +10713,7 @@
       <c r="K372" t="inlineStr"/>
     </row>
     <row r="373">
-      <c r="A373" s="2" t="n">
+      <c r="A373" s="1" t="n">
         <v>42369</v>
       </c>
       <c r="B373" t="n">
@@ -10760,7 +10746,7 @@
       <c r="K373" t="inlineStr"/>
     </row>
     <row r="374">
-      <c r="A374" s="2" t="n">
+      <c r="A374" s="1" t="n">
         <v>42400</v>
       </c>
       <c r="B374" t="inlineStr"/>
@@ -10791,7 +10777,7 @@
       <c r="K374" t="inlineStr"/>
     </row>
     <row r="375">
-      <c r="A375" s="2" t="n">
+      <c r="A375" s="1" t="n">
         <v>42429</v>
       </c>
       <c r="B375" t="inlineStr"/>
@@ -10822,7 +10808,7 @@
       <c r="K375" t="inlineStr"/>
     </row>
     <row r="376">
-      <c r="A376" s="2" t="n">
+      <c r="A376" s="1" t="n">
         <v>42460</v>
       </c>
       <c r="B376" t="n">
@@ -10855,7 +10841,7 @@
       <c r="K376" t="inlineStr"/>
     </row>
     <row r="377">
-      <c r="A377" s="2" t="n">
+      <c r="A377" s="1" t="n">
         <v>42490</v>
       </c>
       <c r="B377" t="inlineStr"/>
@@ -10886,7 +10872,7 @@
       <c r="K377" t="inlineStr"/>
     </row>
     <row r="378">
-      <c r="A378" s="2" t="n">
+      <c r="A378" s="1" t="n">
         <v>42521</v>
       </c>
       <c r="B378" t="inlineStr"/>
@@ -10917,7 +10903,7 @@
       <c r="K378" t="inlineStr"/>
     </row>
     <row r="379">
-      <c r="A379" s="2" t="n">
+      <c r="A379" s="1" t="n">
         <v>42551</v>
       </c>
       <c r="B379" t="n">
@@ -10950,7 +10936,7 @@
       <c r="K379" t="inlineStr"/>
     </row>
     <row r="380">
-      <c r="A380" s="2" t="n">
+      <c r="A380" s="1" t="n">
         <v>42582</v>
       </c>
       <c r="B380" t="inlineStr"/>
@@ -10981,7 +10967,7 @@
       <c r="K380" t="inlineStr"/>
     </row>
     <row r="381">
-      <c r="A381" s="2" t="n">
+      <c r="A381" s="1" t="n">
         <v>42613</v>
       </c>
       <c r="B381" t="inlineStr"/>
@@ -11012,7 +10998,7 @@
       <c r="K381" t="inlineStr"/>
     </row>
     <row r="382">
-      <c r="A382" s="2" t="n">
+      <c r="A382" s="1" t="n">
         <v>42643</v>
       </c>
       <c r="B382" t="n">
@@ -11045,7 +11031,7 @@
       <c r="K382" t="inlineStr"/>
     </row>
     <row r="383">
-      <c r="A383" s="2" t="n">
+      <c r="A383" s="1" t="n">
         <v>42674</v>
       </c>
       <c r="B383" t="inlineStr"/>
@@ -11076,7 +11062,7 @@
       <c r="K383" t="inlineStr"/>
     </row>
     <row r="384">
-      <c r="A384" s="2" t="n">
+      <c r="A384" s="1" t="n">
         <v>42704</v>
       </c>
       <c r="B384" t="inlineStr"/>
@@ -11107,7 +11093,7 @@
       <c r="K384" t="inlineStr"/>
     </row>
     <row r="385">
-      <c r="A385" s="2" t="n">
+      <c r="A385" s="1" t="n">
         <v>42735</v>
       </c>
       <c r="B385" t="n">
@@ -11140,7 +11126,7 @@
       <c r="K385" t="inlineStr"/>
     </row>
     <row r="386">
-      <c r="A386" s="2" t="n">
+      <c r="A386" s="1" t="n">
         <v>42766</v>
       </c>
       <c r="B386" t="inlineStr"/>
@@ -11171,7 +11157,7 @@
       <c r="K386" t="inlineStr"/>
     </row>
     <row r="387">
-      <c r="A387" s="2" t="n">
+      <c r="A387" s="1" t="n">
         <v>42794</v>
       </c>
       <c r="B387" t="inlineStr"/>
@@ -11202,7 +11188,7 @@
       <c r="K387" t="inlineStr"/>
     </row>
     <row r="388">
-      <c r="A388" s="2" t="n">
+      <c r="A388" s="1" t="n">
         <v>42825</v>
       </c>
       <c r="B388" t="n">
@@ -11235,7 +11221,7 @@
       <c r="K388" t="inlineStr"/>
     </row>
     <row r="389">
-      <c r="A389" s="2" t="n">
+      <c r="A389" s="1" t="n">
         <v>42855</v>
       </c>
       <c r="B389" t="inlineStr"/>
@@ -11266,7 +11252,7 @@
       <c r="K389" t="inlineStr"/>
     </row>
     <row r="390">
-      <c r="A390" s="2" t="n">
+      <c r="A390" s="1" t="n">
         <v>42886</v>
       </c>
       <c r="B390" t="inlineStr"/>
@@ -11297,7 +11283,7 @@
       <c r="K390" t="inlineStr"/>
     </row>
     <row r="391">
-      <c r="A391" s="2" t="n">
+      <c r="A391" s="1" t="n">
         <v>42916</v>
       </c>
       <c r="B391" t="n">
@@ -11330,7 +11316,7 @@
       <c r="K391" t="inlineStr"/>
     </row>
     <row r="392">
-      <c r="A392" s="2" t="n">
+      <c r="A392" s="1" t="n">
         <v>42947</v>
       </c>
       <c r="B392" t="inlineStr"/>
@@ -11361,7 +11347,7 @@
       <c r="K392" t="inlineStr"/>
     </row>
     <row r="393">
-      <c r="A393" s="2" t="n">
+      <c r="A393" s="1" t="n">
         <v>42978</v>
       </c>
       <c r="B393" t="inlineStr"/>
@@ -11392,7 +11378,7 @@
       <c r="K393" t="inlineStr"/>
     </row>
     <row r="394">
-      <c r="A394" s="2" t="n">
+      <c r="A394" s="1" t="n">
         <v>43008</v>
       </c>
       <c r="B394" t="n">
@@ -11425,7 +11411,7 @@
       <c r="K394" t="inlineStr"/>
     </row>
     <row r="395">
-      <c r="A395" s="2" t="n">
+      <c r="A395" s="1" t="n">
         <v>43039</v>
       </c>
       <c r="B395" t="inlineStr"/>
@@ -11456,7 +11442,7 @@
       <c r="K395" t="inlineStr"/>
     </row>
     <row r="396">
-      <c r="A396" s="2" t="n">
+      <c r="A396" s="1" t="n">
         <v>43069</v>
       </c>
       <c r="B396" t="inlineStr"/>
@@ -11487,7 +11473,7 @@
       <c r="K396" t="inlineStr"/>
     </row>
     <row r="397">
-      <c r="A397" s="2" t="n">
+      <c r="A397" s="1" t="n">
         <v>43100</v>
       </c>
       <c r="B397" t="n">
@@ -11520,7 +11506,7 @@
       <c r="K397" t="inlineStr"/>
     </row>
     <row r="398">
-      <c r="A398" s="2" t="n">
+      <c r="A398" s="1" t="n">
         <v>43131</v>
       </c>
       <c r="B398" t="inlineStr"/>
@@ -11551,7 +11537,7 @@
       <c r="K398" t="inlineStr"/>
     </row>
     <row r="399">
-      <c r="A399" s="2" t="n">
+      <c r="A399" s="1" t="n">
         <v>43159</v>
       </c>
       <c r="B399" t="inlineStr"/>
@@ -11582,7 +11568,7 @@
       <c r="K399" t="inlineStr"/>
     </row>
     <row r="400">
-      <c r="A400" s="2" t="n">
+      <c r="A400" s="1" t="n">
         <v>43190</v>
       </c>
       <c r="B400" t="n">
@@ -11615,7 +11601,7 @@
       <c r="K400" t="inlineStr"/>
     </row>
     <row r="401">
-      <c r="A401" s="2" t="n">
+      <c r="A401" s="1" t="n">
         <v>43220</v>
       </c>
       <c r="B401" t="inlineStr"/>
@@ -11646,7 +11632,7 @@
       <c r="K401" t="inlineStr"/>
     </row>
     <row r="402">
-      <c r="A402" s="2" t="n">
+      <c r="A402" s="1" t="n">
         <v>43251</v>
       </c>
       <c r="B402" t="inlineStr"/>
@@ -11677,7 +11663,7 @@
       <c r="K402" t="inlineStr"/>
     </row>
     <row r="403">
-      <c r="A403" s="2" t="n">
+      <c r="A403" s="1" t="n">
         <v>43281</v>
       </c>
       <c r="B403" t="n">
@@ -11710,7 +11696,7 @@
       <c r="K403" t="inlineStr"/>
     </row>
     <row r="404">
-      <c r="A404" s="2" t="n">
+      <c r="A404" s="1" t="n">
         <v>43312</v>
       </c>
       <c r="B404" t="inlineStr"/>
@@ -11741,7 +11727,7 @@
       <c r="K404" t="inlineStr"/>
     </row>
     <row r="405">
-      <c r="A405" s="2" t="n">
+      <c r="A405" s="1" t="n">
         <v>43343</v>
       </c>
       <c r="B405" t="inlineStr"/>
@@ -11772,7 +11758,7 @@
       <c r="K405" t="inlineStr"/>
     </row>
     <row r="406">
-      <c r="A406" s="2" t="n">
+      <c r="A406" s="1" t="n">
         <v>43373</v>
       </c>
       <c r="B406" t="n">
@@ -11805,7 +11791,7 @@
       <c r="K406" t="inlineStr"/>
     </row>
     <row r="407">
-      <c r="A407" s="2" t="n">
+      <c r="A407" s="1" t="n">
         <v>43404</v>
       </c>
       <c r="B407" t="inlineStr"/>
@@ -11836,7 +11822,7 @@
       <c r="K407" t="inlineStr"/>
     </row>
     <row r="408">
-      <c r="A408" s="2" t="n">
+      <c r="A408" s="1" t="n">
         <v>43434</v>
       </c>
       <c r="B408" t="inlineStr"/>
@@ -11867,7 +11853,7 @@
       <c r="K408" t="inlineStr"/>
     </row>
     <row r="409">
-      <c r="A409" s="2" t="n">
+      <c r="A409" s="1" t="n">
         <v>43465</v>
       </c>
       <c r="B409" t="n">
@@ -11900,7 +11886,7 @@
       <c r="K409" t="inlineStr"/>
     </row>
     <row r="410">
-      <c r="A410" s="2" t="n">
+      <c r="A410" s="1" t="n">
         <v>43496</v>
       </c>
       <c r="B410" t="inlineStr"/>
@@ -11931,7 +11917,7 @@
       <c r="K410" t="inlineStr"/>
     </row>
     <row r="411">
-      <c r="A411" s="2" t="n">
+      <c r="A411" s="1" t="n">
         <v>43524</v>
       </c>
       <c r="B411" t="inlineStr"/>
@@ -11962,7 +11948,7 @@
       <c r="K411" t="inlineStr"/>
     </row>
     <row r="412">
-      <c r="A412" s="2" t="n">
+      <c r="A412" s="1" t="n">
         <v>43555</v>
       </c>
       <c r="B412" t="n">
@@ -11995,7 +11981,7 @@
       <c r="K412" t="inlineStr"/>
     </row>
     <row r="413">
-      <c r="A413" s="2" t="n">
+      <c r="A413" s="1" t="n">
         <v>43585</v>
       </c>
       <c r="B413" t="inlineStr"/>
@@ -12026,7 +12012,7 @@
       <c r="K413" t="inlineStr"/>
     </row>
     <row r="414">
-      <c r="A414" s="2" t="n">
+      <c r="A414" s="1" t="n">
         <v>43616</v>
       </c>
       <c r="B414" t="inlineStr"/>
@@ -12057,7 +12043,7 @@
       <c r="K414" t="inlineStr"/>
     </row>
     <row r="415">
-      <c r="A415" s="2" t="n">
+      <c r="A415" s="1" t="n">
         <v>43646</v>
       </c>
       <c r="B415" t="n">
@@ -12090,7 +12076,7 @@
       <c r="K415" t="inlineStr"/>
     </row>
     <row r="416">
-      <c r="A416" s="2" t="n">
+      <c r="A416" s="1" t="n">
         <v>43677</v>
       </c>
       <c r="B416" t="inlineStr"/>
@@ -12121,7 +12107,7 @@
       <c r="K416" t="inlineStr"/>
     </row>
     <row r="417">
-      <c r="A417" s="2" t="n">
+      <c r="A417" s="1" t="n">
         <v>43708</v>
       </c>
       <c r="B417" t="inlineStr"/>
@@ -12152,7 +12138,7 @@
       <c r="K417" t="inlineStr"/>
     </row>
     <row r="418">
-      <c r="A418" s="2" t="n">
+      <c r="A418" s="1" t="n">
         <v>43738</v>
       </c>
       <c r="B418" t="n">
@@ -12185,7 +12171,7 @@
       <c r="K418" t="inlineStr"/>
     </row>
     <row r="419">
-      <c r="A419" s="2" t="n">
+      <c r="A419" s="1" t="n">
         <v>43769</v>
       </c>
       <c r="B419" t="inlineStr"/>
@@ -12216,7 +12202,7 @@
       <c r="K419" t="inlineStr"/>
     </row>
     <row r="420">
-      <c r="A420" s="2" t="n">
+      <c r="A420" s="1" t="n">
         <v>43799</v>
       </c>
       <c r="B420" t="inlineStr"/>
@@ -12247,7 +12233,7 @@
       <c r="K420" t="inlineStr"/>
     </row>
     <row r="421">
-      <c r="A421" s="2" t="n">
+      <c r="A421" s="1" t="n">
         <v>43830</v>
       </c>
       <c r="B421" t="n">
@@ -12280,7 +12266,7 @@
       <c r="K421" t="inlineStr"/>
     </row>
     <row r="422">
-      <c r="A422" s="2" t="n">
+      <c r="A422" s="1" t="n">
         <v>43861</v>
       </c>
       <c r="B422" t="inlineStr"/>
@@ -12311,7 +12297,7 @@
       <c r="K422" t="inlineStr"/>
     </row>
     <row r="423">
-      <c r="A423" s="2" t="n">
+      <c r="A423" s="1" t="n">
         <v>43890</v>
       </c>
       <c r="B423" t="inlineStr"/>
@@ -12342,7 +12328,7 @@
       <c r="K423" t="inlineStr"/>
     </row>
     <row r="424">
-      <c r="A424" s="2" t="n">
+      <c r="A424" s="1" t="n">
         <v>43921</v>
       </c>
       <c r="B424" t="n">
@@ -12375,7 +12361,7 @@
       <c r="K424" t="inlineStr"/>
     </row>
     <row r="425">
-      <c r="A425" s="2" t="n">
+      <c r="A425" s="1" t="n">
         <v>43951</v>
       </c>
       <c r="B425" t="inlineStr"/>
@@ -12406,7 +12392,7 @@
       <c r="K425" t="inlineStr"/>
     </row>
     <row r="426">
-      <c r="A426" s="2" t="n">
+      <c r="A426" s="1" t="n">
         <v>43982</v>
       </c>
       <c r="B426" t="inlineStr"/>
@@ -12437,7 +12423,7 @@
       <c r="K426" t="inlineStr"/>
     </row>
     <row r="427">
-      <c r="A427" s="2" t="n">
+      <c r="A427" s="1" t="n">
         <v>44012</v>
       </c>
       <c r="B427" t="n">
@@ -12470,7 +12456,7 @@
       <c r="K427" t="inlineStr"/>
     </row>
     <row r="428">
-      <c r="A428" s="2" t="n">
+      <c r="A428" s="1" t="n">
         <v>44043</v>
       </c>
       <c r="B428" t="inlineStr"/>
@@ -12501,7 +12487,7 @@
       <c r="K428" t="inlineStr"/>
     </row>
     <row r="429">
-      <c r="A429" s="2" t="n">
+      <c r="A429" s="1" t="n">
         <v>44074</v>
       </c>
       <c r="B429" t="inlineStr"/>
@@ -12532,7 +12518,7 @@
       <c r="K429" t="inlineStr"/>
     </row>
     <row r="430">
-      <c r="A430" s="2" t="n">
+      <c r="A430" s="1" t="n">
         <v>44104</v>
       </c>
       <c r="B430" t="n">
@@ -12565,7 +12551,7 @@
       <c r="K430" t="inlineStr"/>
     </row>
     <row r="431">
-      <c r="A431" s="2" t="n">
+      <c r="A431" s="1" t="n">
         <v>44135</v>
       </c>
       <c r="B431" t="inlineStr"/>
@@ -12596,7 +12582,7 @@
       <c r="K431" t="inlineStr"/>
     </row>
     <row r="432">
-      <c r="A432" s="2" t="n">
+      <c r="A432" s="1" t="n">
         <v>44165</v>
       </c>
       <c r="B432" t="inlineStr"/>
@@ -12627,7 +12613,7 @@
       <c r="K432" t="inlineStr"/>
     </row>
     <row r="433">
-      <c r="A433" s="2" t="n">
+      <c r="A433" s="1" t="n">
         <v>44196</v>
       </c>
       <c r="B433" t="n">
@@ -12660,7 +12646,7 @@
       <c r="K433" t="inlineStr"/>
     </row>
     <row r="434">
-      <c r="A434" s="2" t="n">
+      <c r="A434" s="1" t="n">
         <v>44227</v>
       </c>
       <c r="B434" t="inlineStr"/>
@@ -12691,7 +12677,7 @@
       <c r="K434" t="inlineStr"/>
     </row>
     <row r="435">
-      <c r="A435" s="2" t="n">
+      <c r="A435" s="1" t="n">
         <v>44255</v>
       </c>
       <c r="B435" t="inlineStr"/>
@@ -12722,7 +12708,7 @@
       <c r="K435" t="inlineStr"/>
     </row>
     <row r="436">
-      <c r="A436" s="2" t="n">
+      <c r="A436" s="1" t="n">
         <v>44286</v>
       </c>
       <c r="B436" t="n">
@@ -12755,7 +12741,7 @@
       <c r="K436" t="inlineStr"/>
     </row>
     <row r="437">
-      <c r="A437" s="2" t="n">
+      <c r="A437" s="1" t="n">
         <v>44316</v>
       </c>
       <c r="B437" t="inlineStr"/>
@@ -12786,7 +12772,7 @@
       <c r="K437" t="inlineStr"/>
     </row>
     <row r="438">
-      <c r="A438" s="2" t="n">
+      <c r="A438" s="1" t="n">
         <v>44347</v>
       </c>
       <c r="B438" t="inlineStr"/>
@@ -12817,7 +12803,7 @@
       <c r="K438" t="inlineStr"/>
     </row>
     <row r="439">
-      <c r="A439" s="2" t="n">
+      <c r="A439" s="1" t="n">
         <v>44377</v>
       </c>
       <c r="B439" t="n">
@@ -12850,7 +12836,7 @@
       <c r="K439" t="inlineStr"/>
     </row>
     <row r="440">
-      <c r="A440" s="2" t="n">
+      <c r="A440" s="1" t="n">
         <v>44408</v>
       </c>
       <c r="B440" t="inlineStr"/>
@@ -12881,7 +12867,7 @@
       <c r="K440" t="inlineStr"/>
     </row>
     <row r="441">
-      <c r="A441" s="2" t="n">
+      <c r="A441" s="1" t="n">
         <v>44439</v>
       </c>
       <c r="B441" t="inlineStr"/>
@@ -12912,7 +12898,7 @@
       <c r="K441" t="inlineStr"/>
     </row>
     <row r="442">
-      <c r="A442" s="2" t="n">
+      <c r="A442" s="1" t="n">
         <v>44469</v>
       </c>
       <c r="B442" t="n">
@@ -12945,7 +12931,7 @@
       <c r="K442" t="inlineStr"/>
     </row>
     <row r="443">
-      <c r="A443" s="2" t="n">
+      <c r="A443" s="1" t="n">
         <v>44500</v>
       </c>
       <c r="B443" t="inlineStr"/>
@@ -12976,7 +12962,7 @@
       <c r="K443" t="inlineStr"/>
     </row>
     <row r="444">
-      <c r="A444" s="2" t="n">
+      <c r="A444" s="1" t="n">
         <v>44530</v>
       </c>
       <c r="B444" t="inlineStr"/>
@@ -13007,7 +12993,7 @@
       <c r="K444" t="inlineStr"/>
     </row>
     <row r="445">
-      <c r="A445" s="2" t="n">
+      <c r="A445" s="1" t="n">
         <v>44561</v>
       </c>
       <c r="B445" t="n">
@@ -13040,7 +13026,7 @@
       <c r="K445" t="inlineStr"/>
     </row>
     <row r="446">
-      <c r="A446" s="2" t="n">
+      <c r="A446" s="1" t="n">
         <v>44592</v>
       </c>
       <c r="B446" t="inlineStr"/>
@@ -13071,7 +13057,7 @@
       <c r="K446" t="inlineStr"/>
     </row>
     <row r="447">
-      <c r="A447" s="2" t="n">
+      <c r="A447" s="1" t="n">
         <v>44620</v>
       </c>
       <c r="B447" t="inlineStr"/>
@@ -13102,7 +13088,7 @@
       <c r="K447" t="inlineStr"/>
     </row>
     <row r="448">
-      <c r="A448" s="2" t="n">
+      <c r="A448" s="1" t="n">
         <v>44651</v>
       </c>
       <c r="B448" t="n">
@@ -13135,7 +13121,7 @@
       <c r="K448" t="inlineStr"/>
     </row>
     <row r="449">
-      <c r="A449" s="2" t="n">
+      <c r="A449" s="1" t="n">
         <v>44681</v>
       </c>
       <c r="B449" t="inlineStr"/>
@@ -13166,7 +13152,7 @@
       <c r="K449" t="inlineStr"/>
     </row>
     <row r="450">
-      <c r="A450" s="2" t="n">
+      <c r="A450" s="1" t="n">
         <v>44712</v>
       </c>
       <c r="B450" t="inlineStr"/>
@@ -13197,7 +13183,7 @@
       <c r="K450" t="inlineStr"/>
     </row>
     <row r="451">
-      <c r="A451" s="2" t="n">
+      <c r="A451" s="1" t="n">
         <v>44742</v>
       </c>
       <c r="B451" t="n">
@@ -13230,7 +13216,7 @@
       <c r="K451" t="inlineStr"/>
     </row>
     <row r="452">
-      <c r="A452" s="2" t="n">
+      <c r="A452" s="1" t="n">
         <v>44773</v>
       </c>
       <c r="B452" t="inlineStr"/>
@@ -13261,7 +13247,7 @@
       <c r="K452" t="inlineStr"/>
     </row>
     <row r="453">
-      <c r="A453" s="2" t="n">
+      <c r="A453" s="1" t="n">
         <v>44804</v>
       </c>
       <c r="B453" t="inlineStr"/>
@@ -13292,7 +13278,7 @@
       <c r="K453" t="inlineStr"/>
     </row>
     <row r="454">
-      <c r="A454" s="2" t="n">
+      <c r="A454" s="1" t="n">
         <v>44834</v>
       </c>
       <c r="B454" t="n">
@@ -13325,7 +13311,7 @@
       <c r="K454" t="inlineStr"/>
     </row>
     <row r="455">
-      <c r="A455" s="2" t="n">
+      <c r="A455" s="1" t="n">
         <v>44865</v>
       </c>
       <c r="B455" t="inlineStr"/>
@@ -13356,7 +13342,7 @@
       <c r="K455" t="inlineStr"/>
     </row>
     <row r="456">
-      <c r="A456" s="2" t="n">
+      <c r="A456" s="1" t="n">
         <v>44895</v>
       </c>
       <c r="B456" t="inlineStr"/>
@@ -13387,7 +13373,7 @@
       <c r="K456" t="inlineStr"/>
     </row>
     <row r="457">
-      <c r="A457" s="2" t="n">
+      <c r="A457" s="1" t="n">
         <v>44926</v>
       </c>
       <c r="B457" t="n">
@@ -13420,7 +13406,7 @@
       <c r="K457" t="inlineStr"/>
     </row>
     <row r="458">
-      <c r="A458" s="2" t="n">
+      <c r="A458" s="1" t="n">
         <v>44957</v>
       </c>
       <c r="B458" t="inlineStr"/>
@@ -13451,7 +13437,7 @@
       <c r="K458" t="inlineStr"/>
     </row>
     <row r="459">
-      <c r="A459" s="2" t="n">
+      <c r="A459" s="1" t="n">
         <v>44985</v>
       </c>
       <c r="B459" t="inlineStr"/>
@@ -13482,7 +13468,7 @@
       <c r="K459" t="inlineStr"/>
     </row>
     <row r="460">
-      <c r="A460" s="2" t="n">
+      <c r="A460" s="1" t="n">
         <v>45016</v>
       </c>
       <c r="B460" t="n">
@@ -13515,7 +13501,7 @@
       <c r="K460" t="inlineStr"/>
     </row>
     <row r="461">
-      <c r="A461" s="2" t="n">
+      <c r="A461" s="1" t="n">
         <v>45046</v>
       </c>
       <c r="B461" t="inlineStr"/>
@@ -13546,7 +13532,7 @@
       <c r="K461" t="inlineStr"/>
     </row>
     <row r="462">
-      <c r="A462" s="2" t="n">
+      <c r="A462" s="1" t="n">
         <v>45077</v>
       </c>
       <c r="B462" t="inlineStr"/>
@@ -13577,7 +13563,7 @@
       <c r="K462" t="inlineStr"/>
     </row>
     <row r="463">
-      <c r="A463" s="2" t="n">
+      <c r="A463" s="1" t="n">
         <v>45107</v>
       </c>
       <c r="B463" t="n">
@@ -13610,7 +13596,7 @@
       <c r="K463" t="inlineStr"/>
     </row>
     <row r="464">
-      <c r="A464" s="2" t="n">
+      <c r="A464" s="1" t="n">
         <v>45138</v>
       </c>
       <c r="B464" t="inlineStr"/>
@@ -13641,7 +13627,7 @@
       <c r="K464" t="inlineStr"/>
     </row>
     <row r="465">
-      <c r="A465" s="2" t="n">
+      <c r="A465" s="1" t="n">
         <v>45169</v>
       </c>
       <c r="B465" t="inlineStr"/>
@@ -13672,7 +13658,7 @@
       <c r="K465" t="inlineStr"/>
     </row>
     <row r="466">
-      <c r="A466" s="2" t="n">
+      <c r="A466" s="1" t="n">
         <v>45199</v>
       </c>
       <c r="B466" t="n">
@@ -13705,7 +13691,7 @@
       <c r="K466" t="inlineStr"/>
     </row>
     <row r="467">
-      <c r="A467" s="2" t="n">
+      <c r="A467" s="1" t="n">
         <v>45230</v>
       </c>
       <c r="B467" t="inlineStr"/>
@@ -13736,7 +13722,7 @@
       <c r="K467" t="inlineStr"/>
     </row>
     <row r="468">
-      <c r="A468" s="2" t="n">
+      <c r="A468" s="1" t="n">
         <v>45260</v>
       </c>
       <c r="B468" t="inlineStr"/>
@@ -13767,7 +13753,7 @@
       <c r="K468" t="inlineStr"/>
     </row>
     <row r="469">
-      <c r="A469" s="2" t="n">
+      <c r="A469" s="1" t="n">
         <v>45291</v>
       </c>
       <c r="B469" t="n">
@@ -13800,7 +13786,7 @@
       <c r="K469" t="inlineStr"/>
     </row>
     <row r="470">
-      <c r="A470" s="2" t="n">
+      <c r="A470" s="1" t="n">
         <v>45322</v>
       </c>
       <c r="B470" t="inlineStr"/>
@@ -13831,7 +13817,7 @@
       <c r="K470" t="inlineStr"/>
     </row>
     <row r="471">
-      <c r="A471" s="2" t="n">
+      <c r="A471" s="1" t="n">
         <v>45351</v>
       </c>
       <c r="B471" t="inlineStr"/>
@@ -13862,7 +13848,7 @@
       <c r="K471" t="inlineStr"/>
     </row>
     <row r="472">
-      <c r="A472" s="2" t="n">
+      <c r="A472" s="1" t="n">
         <v>45382</v>
       </c>
       <c r="B472" t="n">
@@ -13895,7 +13881,7 @@
       <c r="K472" t="inlineStr"/>
     </row>
     <row r="473">
-      <c r="A473" s="2" t="n">
+      <c r="A473" s="1" t="n">
         <v>45412</v>
       </c>
       <c r="B473" t="inlineStr"/>
@@ -13926,7 +13912,7 @@
       <c r="K473" t="inlineStr"/>
     </row>
     <row r="474">
-      <c r="A474" s="2" t="n">
+      <c r="A474" s="1" t="n">
         <v>45443</v>
       </c>
       <c r="B474" t="inlineStr"/>
@@ -13957,7 +13943,7 @@
       <c r="K474" t="inlineStr"/>
     </row>
     <row r="475">
-      <c r="A475" s="2" t="n">
+      <c r="A475" s="1" t="n">
         <v>45473</v>
       </c>
       <c r="B475" t="n">
@@ -13990,7 +13976,7 @@
       <c r="K475" t="inlineStr"/>
     </row>
     <row r="476">
-      <c r="A476" s="2" t="n">
+      <c r="A476" s="1" t="n">
         <v>45504</v>
       </c>
       <c r="B476" t="inlineStr"/>
@@ -14021,7 +14007,7 @@
       <c r="K476" t="inlineStr"/>
     </row>
     <row r="477">
-      <c r="A477" s="2" t="n">
+      <c r="A477" s="1" t="n">
         <v>45535</v>
       </c>
       <c r="B477" t="inlineStr"/>
@@ -14052,7 +14038,7 @@
       <c r="K477" t="inlineStr"/>
     </row>
     <row r="478">
-      <c r="A478" s="2" t="n">
+      <c r="A478" s="1" t="n">
         <v>45565</v>
       </c>
       <c r="B478" t="n">
@@ -14085,7 +14071,7 @@
       <c r="K478" t="inlineStr"/>
     </row>
     <row r="479">
-      <c r="A479" s="2" t="n">
+      <c r="A479" s="1" t="n">
         <v>45596</v>
       </c>
       <c r="B479" t="inlineStr"/>
@@ -14116,7 +14102,7 @@
       <c r="K479" t="inlineStr"/>
     </row>
     <row r="480">
-      <c r="A480" s="2" t="n">
+      <c r="A480" s="1" t="n">
         <v>45626</v>
       </c>
       <c r="B480" t="inlineStr"/>
@@ -14147,7 +14133,7 @@
       <c r="K480" t="inlineStr"/>
     </row>
     <row r="481">
-      <c r="A481" s="2" t="n">
+      <c r="A481" s="1" t="n">
         <v>45657</v>
       </c>
       <c r="B481" t="n">
@@ -14180,7 +14166,7 @@
       <c r="K481" t="inlineStr"/>
     </row>
     <row r="482">
-      <c r="A482" s="2" t="n">
+      <c r="A482" s="1" t="n">
         <v>45688</v>
       </c>
       <c r="B482" t="inlineStr"/>
@@ -14211,7 +14197,7 @@
       <c r="K482" t="inlineStr"/>
     </row>
     <row r="483">
-      <c r="A483" s="2" t="n">
+      <c r="A483" s="1" t="n">
         <v>45716</v>
       </c>
       <c r="B483" t="inlineStr"/>
@@ -14242,7 +14228,7 @@
       <c r="K483" t="inlineStr"/>
     </row>
     <row r="484">
-      <c r="A484" s="2" t="n">
+      <c r="A484" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="B484" t="n">
@@ -14275,7 +14261,7 @@
       <c r="K484" t="inlineStr"/>
     </row>
     <row r="485">
-      <c r="A485" s="2" t="n">
+      <c r="A485" s="1" t="n">
         <v>45777</v>
       </c>
       <c r="B485" t="inlineStr"/>
@@ -14306,7 +14292,7 @@
       <c r="K485" t="inlineStr"/>
     </row>
     <row r="486">
-      <c r="A486" s="2" t="n">
+      <c r="A486" s="1" t="n">
         <v>45808</v>
       </c>
       <c r="B486" t="inlineStr"/>
@@ -14337,7 +14323,7 @@
       <c r="K486" t="inlineStr"/>
     </row>
     <row r="487">
-      <c r="A487" s="2" t="n">
+      <c r="A487" s="1" t="n">
         <v>45838</v>
       </c>
       <c r="B487" t="n">
@@ -14370,7 +14356,7 @@
       <c r="K487" t="inlineStr"/>
     </row>
     <row r="488">
-      <c r="A488" s="2" t="n">
+      <c r="A488" s="1" t="n">
         <v>45869</v>
       </c>
       <c r="B488" t="inlineStr"/>
@@ -14401,7 +14387,7 @@
       <c r="K488" t="inlineStr"/>
     </row>
     <row r="489">
-      <c r="A489" s="2" t="n">
+      <c r="A489" s="1" t="n">
         <v>45900</v>
       </c>
       <c r="B489" t="inlineStr"/>
@@ -14432,7 +14418,7 @@
       <c r="K489" t="inlineStr"/>
     </row>
     <row r="490">
-      <c r="A490" s="2" t="n">
+      <c r="A490" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="B490" t="n">
@@ -14465,7 +14451,7 @@
       <c r="K490" t="inlineStr"/>
     </row>
     <row r="491">
-      <c r="A491" s="2" t="n">
+      <c r="A491" s="1" t="n">
         <v>45961</v>
       </c>
       <c r="B491" t="inlineStr"/>
@@ -14496,7 +14482,7 @@
       <c r="K491" t="inlineStr"/>
     </row>
     <row r="492">
-      <c r="A492" s="2" t="n">
+      <c r="A492" s="1" t="n">
         <v>45991</v>
       </c>
       <c r="B492" t="inlineStr"/>
@@ -14527,7 +14513,7 @@
       <c r="K492" t="inlineStr"/>
     </row>
     <row r="493">
-      <c r="A493" s="2" t="n">
+      <c r="A493" s="1" t="n">
         <v>46022</v>
       </c>
       <c r="B493" t="n">
@@ -14560,7 +14546,7 @@
       <c r="K493" t="inlineStr"/>
     </row>
     <row r="494">
-      <c r="A494" s="2" t="n">
+      <c r="A494" s="1" t="n">
         <v>46053</v>
       </c>
       <c r="B494" t="inlineStr"/>
@@ -14591,7 +14577,7 @@
       <c r="K494" t="inlineStr"/>
     </row>
     <row r="495">
-      <c r="A495" s="2" t="n">
+      <c r="A495" s="1" t="n">
         <v>46081</v>
       </c>
       <c r="B495" t="inlineStr"/>
@@ -14622,7 +14608,7 @@
       <c r="K495" t="inlineStr"/>
     </row>
     <row r="496">
-      <c r="A496" s="2" t="n">
+      <c r="A496" s="1" t="n">
         <v>46112</v>
       </c>
       <c r="B496" t="n">
@@ -14655,7 +14641,7 @@
       <c r="K496" t="inlineStr"/>
     </row>
     <row r="497">
-      <c r="A497" s="2" t="n">
+      <c r="A497" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="B497" t="inlineStr"/>
@@ -14686,7 +14672,7 @@
       <c r="K497" t="inlineStr"/>
     </row>
     <row r="498">
-      <c r="A498" s="2" t="n">
+      <c r="A498" s="1" t="n">
         <v>46173</v>
       </c>
       <c r="B498" t="inlineStr"/>
@@ -14717,7 +14703,7 @@
       <c r="K498" t="inlineStr"/>
     </row>
     <row r="499">
-      <c r="A499" s="2" t="n">
+      <c r="A499" s="1" t="n">
         <v>46203</v>
       </c>
       <c r="B499" t="n">
@@ -14750,7 +14736,7 @@
       <c r="K499" t="inlineStr"/>
     </row>
     <row r="500">
-      <c r="A500" s="2" t="n">
+      <c r="A500" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="B500" t="inlineStr"/>
@@ -14781,7 +14767,7 @@
       <c r="K500" t="inlineStr"/>
     </row>
     <row r="501">
-      <c r="A501" s="2" t="n">
+      <c r="A501" s="1" t="n">
         <v>46265</v>
       </c>
       <c r="B501" t="inlineStr"/>
@@ -14812,7 +14798,7 @@
       <c r="K501" t="inlineStr"/>
     </row>
     <row r="502">
-      <c r="A502" s="2" t="n">
+      <c r="A502" s="1" t="n">
         <v>46295</v>
       </c>
       <c r="B502" t="inlineStr"/>

</xml_diff>